<commit_message>
Added chapter 5 for merging issues
</commit_message>
<xml_diff>
--- a/PMBOK_ITTOs_Interactive_Dashboard_2025-09-12.xlsx
+++ b/PMBOK_ITTOs_Interactive_Dashboard_2025-09-12.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eric.hayes\Documents\PMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A30E2EA7-97E7-4A39-812B-2C4283184017}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA777300-5A7D-4F72-A34F-CE404B349F0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17565" yWindow="-16320" windowWidth="29040" windowHeight="16440" firstSheet="6" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17565" yWindow="-16320" windowWidth="29040" windowHeight="16440" firstSheet="6" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Interactive Dashboard" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6096" uniqueCount="569">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6120" uniqueCount="569">
   <si>
     <t>Process</t>
   </si>
@@ -2022,12 +2022,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="27">
@@ -2349,7 +2355,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2364,6 +2370,116 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -2407,121 +2523,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -19375,7 +19384,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2795C6F5-9037-7B4A-908E-8E1EB7796907}">
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="3"/>
@@ -19394,148 +19403,233 @@
       <c r="A2" s="3">
         <v>1</v>
       </c>
+      <c r="B2" s="61" t="s">
+        <v>489</v>
+      </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>2</v>
       </c>
+      <c r="B3" s="61" t="s">
+        <v>489</v>
+      </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>3</v>
       </c>
+      <c r="B4" s="61" t="s">
+        <v>489</v>
+      </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>4</v>
       </c>
+      <c r="B5" s="62" t="s">
+        <v>489</v>
+      </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>5</v>
       </c>
+      <c r="B6" s="61" t="s">
+        <v>488</v>
+      </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>6</v>
       </c>
+      <c r="B7" s="61" t="s">
+        <v>487</v>
+      </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>7</v>
       </c>
+      <c r="B8" s="61" t="s">
+        <v>486</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>8</v>
       </c>
+      <c r="B9" s="61" t="s">
+        <v>489</v>
+      </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>9</v>
       </c>
+      <c r="B10" s="61" t="s">
+        <v>488</v>
+      </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>10</v>
+      </c>
+      <c r="B11" s="61" t="s">
+        <v>487</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>11</v>
       </c>
+      <c r="B12" s="61" t="s">
+        <v>487</v>
+      </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
         <v>12</v>
       </c>
+      <c r="B13" s="62" t="s">
+        <v>486</v>
+      </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>13</v>
       </c>
+      <c r="B14" s="62" t="s">
+        <v>487</v>
+      </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
         <v>14</v>
       </c>
+      <c r="B15" s="61" t="s">
+        <v>486</v>
+      </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B16" s="62" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B17" s="61" t="s">
+        <v>488</v>
+      </c>
+      <c r="C17" s="61"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B18" s="62" t="s">
+        <v>488</v>
+      </c>
+      <c r="C18" s="61"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B19" s="61" t="s">
+        <v>487</v>
+      </c>
+      <c r="C19" s="61"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B20" s="61" t="s">
+        <v>489</v>
+      </c>
+      <c r="C20" s="61"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B21" s="61" t="s">
+        <v>489</v>
+      </c>
+      <c r="C21" s="61"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B22" s="61" t="s">
+        <v>486</v>
+      </c>
+      <c r="C22" s="61"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>22</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B23" s="61" t="s">
+        <v>488</v>
+      </c>
+      <c r="C23" s="61"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
         <v>23</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B24" s="61" t="s">
+        <v>487</v>
+      </c>
+      <c r="C24" s="61"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
         <v>24</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B25" s="61" t="s">
+        <v>487</v>
+      </c>
+      <c r="C25" s="61"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
         <v>25</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B26" s="61"/>
+      <c r="C26" s="63">
+        <v>0.79166666666666663</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -19582,7 +19676,7 @@
       <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="59" t="s">
+      <c r="B4" s="7" t="s">
         <v>486</v>
       </c>
     </row>
@@ -19590,7 +19684,7 @@
       <c r="A5" s="3">
         <v>4</v>
       </c>
-      <c r="B5" s="59" t="s">
+      <c r="B5" s="7" t="s">
         <v>489</v>
       </c>
     </row>
@@ -19662,7 +19756,7 @@
       <c r="A14" s="3">
         <v>13</v>
       </c>
-      <c r="B14" s="59" t="s">
+      <c r="B14" s="7" t="s">
         <v>486</v>
       </c>
     </row>
@@ -19670,7 +19764,7 @@
       <c r="A15" s="3">
         <v>14</v>
       </c>
-      <c r="B15" s="59" t="s">
+      <c r="B15" s="7" t="s">
         <v>487</v>
       </c>
     </row>
@@ -19678,7 +19772,7 @@
       <c r="A16" s="3">
         <v>15</v>
       </c>
-      <c r="B16" s="59" t="s">
+      <c r="B16" s="7" t="s">
         <v>489</v>
       </c>
     </row>
@@ -19686,7 +19780,7 @@
       <c r="A17" s="3">
         <v>16</v>
       </c>
-      <c r="B17" s="59" t="s">
+      <c r="B17" s="7" t="s">
         <v>486</v>
       </c>
     </row>
@@ -19694,7 +19788,7 @@
       <c r="A18" s="3">
         <v>17</v>
       </c>
-      <c r="B18" s="59" t="s">
+      <c r="B18" s="7" t="s">
         <v>488</v>
       </c>
     </row>
@@ -19726,7 +19820,7 @@
       <c r="A22" s="3">
         <v>21</v>
       </c>
-      <c r="B22" s="59" t="s">
+      <c r="B22" s="7" t="s">
         <v>486</v>
       </c>
     </row>
@@ -19811,7 +19905,7 @@
       <c r="B33" t="s">
         <v>568</v>
       </c>
-      <c r="C33" s="60">
+      <c r="C33" s="8">
         <f>1-(8/31)</f>
         <v>0.74193548387096775</v>
       </c>
@@ -19834,52 +19928,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="50" t="s">
         <v>469</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="51" t="s">
+      <c r="B1" s="51"/>
+      <c r="C1" s="9" t="s">
         <v>470</v>
       </c>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
-      <c r="H1" s="52"/>
-      <c r="I1" s="52"/>
-      <c r="J1" s="52"/>
-      <c r="K1" s="52"/>
-      <c r="L1" s="53"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="11"/>
     </row>
     <row r="2" spans="1:12" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="14"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="54" t="s">
+      <c r="A2" s="52"/>
+      <c r="B2" s="53"/>
+      <c r="C2" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="55"/>
-      <c r="E2" s="54" t="s">
-        <v>57</v>
-      </c>
-      <c r="F2" s="55"/>
-      <c r="G2" s="54" t="s">
+      <c r="D2" s="13"/>
+      <c r="E2" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="13"/>
+      <c r="G2" s="12" t="s">
         <v>249</v>
       </c>
-      <c r="H2" s="55"/>
-      <c r="I2" s="56" t="s">
+      <c r="H2" s="13"/>
+      <c r="I2" s="14" t="s">
         <v>481</v>
       </c>
-      <c r="J2" s="55"/>
-      <c r="K2" s="54" t="s">
+      <c r="J2" s="13"/>
+      <c r="K2" s="12" t="s">
         <v>377</v>
       </c>
-      <c r="L2" s="55"/>
+      <c r="L2" s="13"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="54" t="s">
         <v>471</v>
       </c>
-      <c r="B3" s="17"/>
+      <c r="B3" s="55"/>
       <c r="C3" s="41" t="s">
         <v>7</v>
       </c>
@@ -19888,499 +19982,443 @@
         <v>56</v>
       </c>
       <c r="F3" s="44"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="27"/>
+      <c r="G3" s="38"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="38"/>
+      <c r="J3" s="39"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="40"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A4" s="9"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="35"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="24"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="28"/>
+      <c r="A4" s="47"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="25"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="25"/>
+      <c r="L4" s="30"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A5" s="9"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="25"/>
-      <c r="J5" s="26"/>
-      <c r="K5" s="25"/>
-      <c r="L5" s="29"/>
+      <c r="A5" s="47"/>
+      <c r="B5" s="46"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="28"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="28"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="31"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="56" t="s">
         <v>472</v>
       </c>
-      <c r="B6" s="19"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="32" t="s">
+      <c r="B6" s="57"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="17" t="s">
         <v>482</v>
       </c>
-      <c r="F6" s="33"/>
-      <c r="G6" s="38"/>
-      <c r="H6" s="39"/>
-      <c r="I6" s="38"/>
-      <c r="J6" s="39"/>
-      <c r="K6" s="38"/>
-      <c r="L6" s="40"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="24"/>
+      <c r="K6" s="23"/>
+      <c r="L6" s="29"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A7" s="20"/>
-      <c r="B7" s="19"/>
-      <c r="C7" s="31"/>
-      <c r="D7" s="31"/>
-      <c r="E7" s="34"/>
-      <c r="F7" s="35"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="23"/>
-      <c r="J7" s="24"/>
-      <c r="K7" s="23"/>
-      <c r="L7" s="28"/>
+      <c r="A7" s="58"/>
+      <c r="B7" s="57"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="25"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="25"/>
+      <c r="L7" s="30"/>
     </row>
     <row r="8" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="20"/>
-      <c r="B8" s="19"/>
-      <c r="C8" s="31"/>
-      <c r="D8" s="31"/>
-      <c r="E8" s="36"/>
-      <c r="F8" s="37"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="25"/>
-      <c r="J8" s="26"/>
-      <c r="K8" s="25"/>
-      <c r="L8" s="29"/>
+      <c r="A8" s="58"/>
+      <c r="B8" s="57"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="28"/>
+      <c r="K8" s="27"/>
+      <c r="L8" s="31"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="45" t="s">
         <v>473</v>
       </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="33"/>
-      <c r="G9" s="38"/>
-      <c r="H9" s="39"/>
-      <c r="I9" s="38"/>
-      <c r="J9" s="39"/>
-      <c r="K9" s="38"/>
-      <c r="L9" s="40"/>
+      <c r="B9" s="46"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="24"/>
+      <c r="I9" s="23"/>
+      <c r="J9" s="24"/>
+      <c r="K9" s="23"/>
+      <c r="L9" s="29"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A10" s="9"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="31"/>
-      <c r="D10" s="31"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="23"/>
-      <c r="J10" s="24"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="28"/>
+      <c r="A10" s="47"/>
+      <c r="B10" s="46"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="25"/>
+      <c r="J10" s="26"/>
+      <c r="K10" s="25"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A11" s="9"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="31"/>
-      <c r="E11" s="36"/>
-      <c r="F11" s="37"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="25"/>
-      <c r="J11" s="26"/>
-      <c r="K11" s="25"/>
-      <c r="L11" s="29"/>
+      <c r="A11" s="47"/>
+      <c r="B11" s="46"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="28"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="28"/>
+      <c r="K11" s="27"/>
+      <c r="L11" s="31"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="45" t="s">
         <v>474</v>
       </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="31"/>
-      <c r="E12" s="32"/>
-      <c r="F12" s="33"/>
-      <c r="G12" s="38"/>
-      <c r="H12" s="39"/>
-      <c r="I12" s="38"/>
-      <c r="J12" s="39"/>
-      <c r="K12" s="38"/>
-      <c r="L12" s="40"/>
+      <c r="B12" s="46"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="23"/>
+      <c r="J12" s="24"/>
+      <c r="K12" s="23"/>
+      <c r="L12" s="29"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A13" s="9"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="31"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="23"/>
-      <c r="H13" s="24"/>
-      <c r="I13" s="23"/>
-      <c r="J13" s="24"/>
-      <c r="K13" s="23"/>
-      <c r="L13" s="28"/>
+      <c r="A13" s="47"/>
+      <c r="B13" s="46"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="25"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="25"/>
+      <c r="J13" s="26"/>
+      <c r="K13" s="25"/>
+      <c r="L13" s="30"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A14" s="9"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="31"/>
-      <c r="D14" s="31"/>
-      <c r="E14" s="36"/>
-      <c r="F14" s="37"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="25"/>
-      <c r="J14" s="26"/>
-      <c r="K14" s="25"/>
-      <c r="L14" s="29"/>
+      <c r="A14" s="47"/>
+      <c r="B14" s="46"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="28"/>
+      <c r="K14" s="27"/>
+      <c r="L14" s="31"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="45" t="s">
         <v>475</v>
       </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="30"/>
-      <c r="D15" s="31"/>
-      <c r="E15" s="32"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="38"/>
-      <c r="H15" s="39"/>
-      <c r="I15" s="38"/>
-      <c r="J15" s="39"/>
-      <c r="K15" s="38"/>
-      <c r="L15" s="40"/>
+      <c r="B15" s="46"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="24"/>
+      <c r="I15" s="23"/>
+      <c r="J15" s="24"/>
+      <c r="K15" s="23"/>
+      <c r="L15" s="29"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A16" s="9"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="31"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="35"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="24"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="24"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="28"/>
+      <c r="A16" s="47"/>
+      <c r="B16" s="46"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="26"/>
+      <c r="I16" s="25"/>
+      <c r="J16" s="26"/>
+      <c r="K16" s="25"/>
+      <c r="L16" s="30"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A17" s="9"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="31"/>
-      <c r="D17" s="31"/>
-      <c r="E17" s="36"/>
-      <c r="F17" s="37"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="26"/>
-      <c r="I17" s="25"/>
-      <c r="J17" s="26"/>
-      <c r="K17" s="25"/>
-      <c r="L17" s="29"/>
+      <c r="A17" s="47"/>
+      <c r="B17" s="46"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="28"/>
+      <c r="I17" s="27"/>
+      <c r="J17" s="28"/>
+      <c r="K17" s="27"/>
+      <c r="L17" s="31"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="45" t="s">
         <v>476</v>
       </c>
-      <c r="B18" s="8"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="33"/>
-      <c r="G18" s="38"/>
-      <c r="H18" s="39"/>
-      <c r="I18" s="38"/>
-      <c r="J18" s="39"/>
-      <c r="K18" s="38"/>
-      <c r="L18" s="40"/>
+      <c r="B18" s="46"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="23"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="23"/>
+      <c r="L18" s="29"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A19" s="9"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="35"/>
-      <c r="G19" s="23"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="23"/>
-      <c r="J19" s="24"/>
-      <c r="K19" s="23"/>
-      <c r="L19" s="28"/>
+      <c r="A19" s="47"/>
+      <c r="B19" s="46"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="25"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="25"/>
+      <c r="J19" s="26"/>
+      <c r="K19" s="25"/>
+      <c r="L19" s="30"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A20" s="9"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="31"/>
-      <c r="D20" s="31"/>
-      <c r="E20" s="36"/>
-      <c r="F20" s="37"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="26"/>
-      <c r="I20" s="25"/>
-      <c r="J20" s="26"/>
-      <c r="K20" s="25"/>
-      <c r="L20" s="29"/>
+      <c r="A20" s="47"/>
+      <c r="B20" s="46"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="28"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="28"/>
+      <c r="K20" s="27"/>
+      <c r="L20" s="31"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="45" t="s">
         <v>477</v>
       </c>
-      <c r="B21" s="8"/>
-      <c r="C21" s="30"/>
-      <c r="D21" s="31"/>
-      <c r="E21" s="32"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="38"/>
-      <c r="H21" s="39"/>
-      <c r="I21" s="38"/>
-      <c r="J21" s="39"/>
-      <c r="K21" s="38"/>
-      <c r="L21" s="40"/>
+      <c r="B21" s="46"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="23"/>
+      <c r="H21" s="24"/>
+      <c r="I21" s="23"/>
+      <c r="J21" s="24"/>
+      <c r="K21" s="23"/>
+      <c r="L21" s="29"/>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A22" s="9"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="31"/>
-      <c r="D22" s="31"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="35"/>
-      <c r="G22" s="23"/>
-      <c r="H22" s="24"/>
-      <c r="I22" s="23"/>
-      <c r="J22" s="24"/>
-      <c r="K22" s="23"/>
-      <c r="L22" s="28"/>
+      <c r="A22" s="47"/>
+      <c r="B22" s="46"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="25"/>
+      <c r="H22" s="26"/>
+      <c r="I22" s="25"/>
+      <c r="J22" s="26"/>
+      <c r="K22" s="25"/>
+      <c r="L22" s="30"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A23" s="9"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="31"/>
-      <c r="D23" s="31"/>
-      <c r="E23" s="36"/>
-      <c r="F23" s="37"/>
-      <c r="G23" s="25"/>
-      <c r="H23" s="26"/>
-      <c r="I23" s="25"/>
-      <c r="J23" s="26"/>
-      <c r="K23" s="25"/>
-      <c r="L23" s="29"/>
+      <c r="A23" s="47"/>
+      <c r="B23" s="46"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="22"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="28"/>
+      <c r="I23" s="27"/>
+      <c r="J23" s="28"/>
+      <c r="K23" s="27"/>
+      <c r="L23" s="31"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="45" t="s">
         <v>478</v>
       </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="30"/>
-      <c r="D24" s="31"/>
-      <c r="E24" s="32"/>
-      <c r="F24" s="33"/>
-      <c r="G24" s="38"/>
-      <c r="H24" s="39"/>
-      <c r="I24" s="38"/>
-      <c r="J24" s="39"/>
-      <c r="K24" s="38"/>
-      <c r="L24" s="40"/>
+      <c r="B24" s="46"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="18"/>
+      <c r="G24" s="23"/>
+      <c r="H24" s="24"/>
+      <c r="I24" s="23"/>
+      <c r="J24" s="24"/>
+      <c r="K24" s="23"/>
+      <c r="L24" s="29"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A25" s="9"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="31"/>
-      <c r="D25" s="31"/>
-      <c r="E25" s="34"/>
-      <c r="F25" s="35"/>
-      <c r="G25" s="23"/>
-      <c r="H25" s="24"/>
-      <c r="I25" s="23"/>
-      <c r="J25" s="24"/>
-      <c r="K25" s="23"/>
-      <c r="L25" s="28"/>
+      <c r="A25" s="47"/>
+      <c r="B25" s="46"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="25"/>
+      <c r="H25" s="26"/>
+      <c r="I25" s="25"/>
+      <c r="J25" s="26"/>
+      <c r="K25" s="25"/>
+      <c r="L25" s="30"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A26" s="9"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="31"/>
-      <c r="D26" s="31"/>
-      <c r="E26" s="36"/>
-      <c r="F26" s="37"/>
-      <c r="G26" s="25"/>
-      <c r="H26" s="26"/>
-      <c r="I26" s="25"/>
-      <c r="J26" s="26"/>
-      <c r="K26" s="25"/>
-      <c r="L26" s="29"/>
+      <c r="A26" s="47"/>
+      <c r="B26" s="46"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="27"/>
+      <c r="H26" s="28"/>
+      <c r="I26" s="27"/>
+      <c r="J26" s="28"/>
+      <c r="K26" s="27"/>
+      <c r="L26" s="31"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="45" t="s">
         <v>479</v>
       </c>
-      <c r="B27" s="8"/>
-      <c r="C27" s="30"/>
-      <c r="D27" s="31"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="33"/>
-      <c r="G27" s="38"/>
-      <c r="H27" s="39"/>
-      <c r="I27" s="38"/>
-      <c r="J27" s="39"/>
-      <c r="K27" s="38"/>
-      <c r="L27" s="40"/>
+      <c r="B27" s="46"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="23"/>
+      <c r="H27" s="24"/>
+      <c r="I27" s="23"/>
+      <c r="J27" s="24"/>
+      <c r="K27" s="23"/>
+      <c r="L27" s="29"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A28" s="9"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31"/>
-      <c r="E28" s="34"/>
-      <c r="F28" s="35"/>
-      <c r="G28" s="23"/>
-      <c r="H28" s="24"/>
-      <c r="I28" s="23"/>
-      <c r="J28" s="24"/>
-      <c r="K28" s="23"/>
-      <c r="L28" s="28"/>
+      <c r="A28" s="47"/>
+      <c r="B28" s="46"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="26"/>
+      <c r="I28" s="25"/>
+      <c r="J28" s="26"/>
+      <c r="K28" s="25"/>
+      <c r="L28" s="30"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A29" s="9"/>
-      <c r="B29" s="8"/>
-      <c r="C29" s="31"/>
-      <c r="D29" s="31"/>
-      <c r="E29" s="36"/>
-      <c r="F29" s="37"/>
-      <c r="G29" s="25"/>
-      <c r="H29" s="26"/>
-      <c r="I29" s="25"/>
-      <c r="J29" s="26"/>
-      <c r="K29" s="25"/>
-      <c r="L29" s="29"/>
+      <c r="A29" s="47"/>
+      <c r="B29" s="46"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="27"/>
+      <c r="H29" s="28"/>
+      <c r="I29" s="27"/>
+      <c r="J29" s="28"/>
+      <c r="K29" s="27"/>
+      <c r="L29" s="31"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A30" s="7" t="s">
+      <c r="A30" s="45" t="s">
         <v>480</v>
       </c>
-      <c r="B30" s="8"/>
-      <c r="C30" s="30" t="s">
+      <c r="B30" s="46"/>
+      <c r="C30" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="D30" s="31"/>
-      <c r="E30" s="32"/>
-      <c r="F30" s="33"/>
-      <c r="G30" s="38"/>
-      <c r="H30" s="39"/>
-      <c r="I30" s="38"/>
-      <c r="J30" s="39"/>
-      <c r="K30" s="38"/>
-      <c r="L30" s="40"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="23"/>
+      <c r="H30" s="24"/>
+      <c r="I30" s="23"/>
+      <c r="J30" s="24"/>
+      <c r="K30" s="23"/>
+      <c r="L30" s="29"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A31" s="9"/>
-      <c r="B31" s="8"/>
-      <c r="C31" s="31"/>
-      <c r="D31" s="31"/>
-      <c r="E31" s="34"/>
-      <c r="F31" s="35"/>
-      <c r="G31" s="23"/>
-      <c r="H31" s="24"/>
-      <c r="I31" s="23"/>
-      <c r="J31" s="24"/>
-      <c r="K31" s="23"/>
-      <c r="L31" s="28"/>
+      <c r="A31" s="47"/>
+      <c r="B31" s="46"/>
+      <c r="C31" s="16"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="20"/>
+      <c r="G31" s="25"/>
+      <c r="H31" s="26"/>
+      <c r="I31" s="25"/>
+      <c r="J31" s="26"/>
+      <c r="K31" s="25"/>
+      <c r="L31" s="30"/>
     </row>
     <row r="32" spans="1:12" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="10"/>
-      <c r="B32" s="11"/>
-      <c r="C32" s="45"/>
-      <c r="D32" s="45"/>
-      <c r="E32" s="46"/>
-      <c r="F32" s="47"/>
-      <c r="G32" s="48"/>
-      <c r="H32" s="49"/>
-      <c r="I32" s="48"/>
-      <c r="J32" s="49"/>
-      <c r="K32" s="48"/>
-      <c r="L32" s="50"/>
+      <c r="A32" s="48"/>
+      <c r="B32" s="49"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="33"/>
+      <c r="F32" s="34"/>
+      <c r="G32" s="35"/>
+      <c r="H32" s="36"/>
+      <c r="I32" s="35"/>
+      <c r="J32" s="36"/>
+      <c r="K32" s="35"/>
+      <c r="L32" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="67">
-    <mergeCell ref="C1:L1"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="C27:D29"/>
-    <mergeCell ref="E27:F29"/>
-    <mergeCell ref="G27:H29"/>
-    <mergeCell ref="I27:J29"/>
-    <mergeCell ref="K27:L29"/>
-    <mergeCell ref="C30:D32"/>
-    <mergeCell ref="E30:F32"/>
-    <mergeCell ref="G30:H32"/>
-    <mergeCell ref="I30:J32"/>
-    <mergeCell ref="K30:L32"/>
-    <mergeCell ref="C21:D23"/>
-    <mergeCell ref="E21:F23"/>
-    <mergeCell ref="G21:H23"/>
-    <mergeCell ref="I21:J23"/>
-    <mergeCell ref="K21:L23"/>
-    <mergeCell ref="C24:D26"/>
-    <mergeCell ref="E24:F26"/>
-    <mergeCell ref="G24:H26"/>
-    <mergeCell ref="I24:J26"/>
-    <mergeCell ref="K24:L26"/>
-    <mergeCell ref="C15:D17"/>
-    <mergeCell ref="E15:F17"/>
-    <mergeCell ref="G15:H17"/>
-    <mergeCell ref="I15:J17"/>
-    <mergeCell ref="K15:L17"/>
-    <mergeCell ref="C18:D20"/>
-    <mergeCell ref="E18:F20"/>
-    <mergeCell ref="G18:H20"/>
-    <mergeCell ref="I18:J20"/>
-    <mergeCell ref="K18:L20"/>
-    <mergeCell ref="E9:F11"/>
-    <mergeCell ref="G9:H11"/>
-    <mergeCell ref="I9:J11"/>
-    <mergeCell ref="K9:L11"/>
-    <mergeCell ref="C12:D14"/>
-    <mergeCell ref="E12:F14"/>
-    <mergeCell ref="G12:H14"/>
-    <mergeCell ref="I12:J14"/>
-    <mergeCell ref="K12:L14"/>
-    <mergeCell ref="C9:D11"/>
-    <mergeCell ref="I3:J5"/>
-    <mergeCell ref="K3:L5"/>
-    <mergeCell ref="C6:D8"/>
-    <mergeCell ref="E6:F8"/>
-    <mergeCell ref="G6:H8"/>
-    <mergeCell ref="I6:J8"/>
-    <mergeCell ref="K6:L8"/>
-    <mergeCell ref="C3:D5"/>
-    <mergeCell ref="E3:F5"/>
-    <mergeCell ref="G3:H5"/>
     <mergeCell ref="A30:B32"/>
     <mergeCell ref="A1:B2"/>
     <mergeCell ref="A3:B5"/>
@@ -20392,6 +20430,62 @@
     <mergeCell ref="A21:B23"/>
     <mergeCell ref="A24:B26"/>
     <mergeCell ref="A27:B29"/>
+    <mergeCell ref="I3:J5"/>
+    <mergeCell ref="K3:L5"/>
+    <mergeCell ref="C6:D8"/>
+    <mergeCell ref="E6:F8"/>
+    <mergeCell ref="G6:H8"/>
+    <mergeCell ref="I6:J8"/>
+    <mergeCell ref="K6:L8"/>
+    <mergeCell ref="C3:D5"/>
+    <mergeCell ref="E3:F5"/>
+    <mergeCell ref="G3:H5"/>
+    <mergeCell ref="E9:F11"/>
+    <mergeCell ref="G9:H11"/>
+    <mergeCell ref="I9:J11"/>
+    <mergeCell ref="K9:L11"/>
+    <mergeCell ref="C12:D14"/>
+    <mergeCell ref="E12:F14"/>
+    <mergeCell ref="G12:H14"/>
+    <mergeCell ref="I12:J14"/>
+    <mergeCell ref="K12:L14"/>
+    <mergeCell ref="C9:D11"/>
+    <mergeCell ref="C18:D20"/>
+    <mergeCell ref="E18:F20"/>
+    <mergeCell ref="G18:H20"/>
+    <mergeCell ref="I18:J20"/>
+    <mergeCell ref="K18:L20"/>
+    <mergeCell ref="C15:D17"/>
+    <mergeCell ref="E15:F17"/>
+    <mergeCell ref="G15:H17"/>
+    <mergeCell ref="I15:J17"/>
+    <mergeCell ref="K15:L17"/>
+    <mergeCell ref="C24:D26"/>
+    <mergeCell ref="E24:F26"/>
+    <mergeCell ref="G24:H26"/>
+    <mergeCell ref="I24:J26"/>
+    <mergeCell ref="K24:L26"/>
+    <mergeCell ref="C21:D23"/>
+    <mergeCell ref="E21:F23"/>
+    <mergeCell ref="G21:H23"/>
+    <mergeCell ref="I21:J23"/>
+    <mergeCell ref="K21:L23"/>
+    <mergeCell ref="C30:D32"/>
+    <mergeCell ref="E30:F32"/>
+    <mergeCell ref="G30:H32"/>
+    <mergeCell ref="I30:J32"/>
+    <mergeCell ref="K30:L32"/>
+    <mergeCell ref="C27:D29"/>
+    <mergeCell ref="E27:F29"/>
+    <mergeCell ref="G27:H29"/>
+    <mergeCell ref="I27:J29"/>
+    <mergeCell ref="K27:L29"/>
+    <mergeCell ref="C1:L1"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="K2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -28614,183 +28708,183 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="59" t="s">
         <v>483</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A2" s="58"/>
+      <c r="A2" s="60"/>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A3" s="58"/>
+      <c r="A3" s="60"/>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" s="58"/>
+      <c r="A4" s="60"/>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A5" s="58"/>
+      <c r="A5" s="60"/>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A6" s="58"/>
+      <c r="A6" s="60"/>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A7" s="58"/>
+      <c r="A7" s="60"/>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A8" s="58"/>
+      <c r="A8" s="60"/>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A9" s="58"/>
+      <c r="A9" s="60"/>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A10" s="58"/>
+      <c r="A10" s="60"/>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A11" s="58"/>
+      <c r="A11" s="60"/>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A12" s="58"/>
+      <c r="A12" s="60"/>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A13" s="58"/>
+      <c r="A13" s="60"/>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A14" s="58"/>
+      <c r="A14" s="60"/>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A15" s="58"/>
+      <c r="A15" s="60"/>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A16" s="58"/>
+      <c r="A16" s="60"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" s="58"/>
+      <c r="A17" s="60"/>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A18" s="58"/>
+      <c r="A18" s="60"/>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A19" s="58"/>
+      <c r="A19" s="60"/>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A20" s="58"/>
+      <c r="A20" s="60"/>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A21" s="58"/>
+      <c r="A21" s="60"/>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A22" s="58"/>
+      <c r="A22" s="60"/>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A23" s="58"/>
+      <c r="A23" s="60"/>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" s="58"/>
+      <c r="A24" s="60"/>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" s="58"/>
+      <c r="A25" s="60"/>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A26" s="58"/>
+      <c r="A26" s="60"/>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" s="58"/>
+      <c r="A27" s="60"/>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A28" s="58"/>
+      <c r="A28" s="60"/>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A29" s="58"/>
+      <c r="A29" s="60"/>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A30" s="58"/>
+      <c r="A30" s="60"/>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A31" s="58"/>
+      <c r="A31" s="60"/>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A32" s="58"/>
+      <c r="A32" s="60"/>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" s="58"/>
+      <c r="A33" s="60"/>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A34" s="58"/>
+      <c r="A34" s="60"/>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A35" s="58"/>
+      <c r="A35" s="60"/>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A36" s="58"/>
+      <c r="A36" s="60"/>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A37" s="58"/>
+      <c r="A37" s="60"/>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A38" s="58"/>
+      <c r="A38" s="60"/>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A39" s="58"/>
+      <c r="A39" s="60"/>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A40" s="58"/>
+      <c r="A40" s="60"/>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A41" s="58"/>
+      <c r="A41" s="60"/>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A42" s="58"/>
+      <c r="A42" s="60"/>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A43" s="58"/>
+      <c r="A43" s="60"/>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A44" s="58"/>
+      <c r="A44" s="60"/>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A45" s="58"/>
+      <c r="A45" s="60"/>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A46" s="58"/>
+      <c r="A46" s="60"/>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A47" s="58"/>
+      <c r="A47" s="60"/>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A48" s="58"/>
+      <c r="A48" s="60"/>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A49" s="58"/>
+      <c r="A49" s="60"/>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A50" s="58"/>
+      <c r="A50" s="60"/>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A51" s="58"/>
+      <c r="A51" s="60"/>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A52" s="58"/>
+      <c r="A52" s="60"/>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A53" s="58"/>
+      <c r="A53" s="60"/>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A54" s="58"/>
+      <c r="A54" s="60"/>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A55" s="58"/>
+      <c r="A55" s="60"/>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A56" s="58"/>
+      <c r="A56" s="60"/>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A57" s="58"/>
+      <c r="A57" s="60"/>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A58" s="58"/>
+      <c r="A58" s="60"/>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A59" s="58"/>
+      <c r="A59" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Chapter 7 - Schedule completed
</commit_message>
<xml_diff>
--- a/PMBOK_ITTOs_Interactive_Dashboard_2025-09-12.xlsx
+++ b/PMBOK_ITTOs_Interactive_Dashboard_2025-09-12.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eric.hayes\Documents\PMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D01F4DA-34BE-47CC-9B35-8AE188E13562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1167CD95-E36E-4031-8FAA-0F7BE55DBAFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-11235" yWindow="-16395" windowWidth="29040" windowHeight="16440" firstSheet="10" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Definitions" sheetId="16" r:id="rId1"/>
@@ -28,6 +28,7 @@
     <sheet name="CH4 Agile" sheetId="9" r:id="rId13"/>
     <sheet name="CH5 IntegrationMGMT" sheetId="11" r:id="rId14"/>
     <sheet name="CH6 Project Scope Management" sheetId="15" r:id="rId15"/>
+    <sheet name="CH7 Project Schedule Management" sheetId="17" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="Slicer_ITTO_Name">#N/A</definedName>
@@ -41,9 +42,9 @@
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{46BE6895-7355-4a93-B00E-2C351335B9C9}">
       <x15:slicerCaches xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
-        <x14:slicerCache r:id="rId16"/>
         <x14:slicerCache r:id="rId17"/>
         <x14:slicerCache r:id="rId18"/>
+        <x14:slicerCache r:id="rId19"/>
       </x15:slicerCaches>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -62,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6122" uniqueCount="571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6153" uniqueCount="571">
   <si>
     <t>Process</t>
   </si>
@@ -2027,7 +2028,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2069,6 +2070,12 @@
     <font>
       <sz val="12"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2407,7 +2414,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2426,6 +2433,117 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2468,123 +2586,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3247,7 +3255,7 @@
       </c>
     </row>
     <row r="27" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E27" s="62" t="s">
+      <c r="E27" s="10" t="s">
         <v>569</v>
       </c>
     </row>
@@ -3265,183 +3273,183 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="61" t="s">
         <v>483</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A2" s="61"/>
+      <c r="A2" s="62"/>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A3" s="61"/>
+      <c r="A3" s="62"/>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" s="61"/>
+      <c r="A4" s="62"/>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A5" s="61"/>
+      <c r="A5" s="62"/>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A6" s="61"/>
+      <c r="A6" s="62"/>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A7" s="61"/>
+      <c r="A7" s="62"/>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A8" s="61"/>
+      <c r="A8" s="62"/>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A9" s="61"/>
+      <c r="A9" s="62"/>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A10" s="61"/>
+      <c r="A10" s="62"/>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A11" s="61"/>
+      <c r="A11" s="62"/>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A12" s="61"/>
+      <c r="A12" s="62"/>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A13" s="61"/>
+      <c r="A13" s="62"/>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A14" s="61"/>
+      <c r="A14" s="62"/>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A15" s="61"/>
+      <c r="A15" s="62"/>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A16" s="61"/>
+      <c r="A16" s="62"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" s="61"/>
+      <c r="A17" s="62"/>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A18" s="61"/>
+      <c r="A18" s="62"/>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A19" s="61"/>
+      <c r="A19" s="62"/>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A20" s="61"/>
+      <c r="A20" s="62"/>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A21" s="61"/>
+      <c r="A21" s="62"/>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A22" s="61"/>
+      <c r="A22" s="62"/>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A23" s="61"/>
+      <c r="A23" s="62"/>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" s="61"/>
+      <c r="A24" s="62"/>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" s="61"/>
+      <c r="A25" s="62"/>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A26" s="61"/>
+      <c r="A26" s="62"/>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" s="61"/>
+      <c r="A27" s="62"/>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A28" s="61"/>
+      <c r="A28" s="62"/>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A29" s="61"/>
+      <c r="A29" s="62"/>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A30" s="61"/>
+      <c r="A30" s="62"/>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A31" s="61"/>
+      <c r="A31" s="62"/>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A32" s="61"/>
+      <c r="A32" s="62"/>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" s="61"/>
+      <c r="A33" s="62"/>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A34" s="61"/>
+      <c r="A34" s="62"/>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A35" s="61"/>
+      <c r="A35" s="62"/>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A36" s="61"/>
+      <c r="A36" s="62"/>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A37" s="61"/>
+      <c r="A37" s="62"/>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A38" s="61"/>
+      <c r="A38" s="62"/>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A39" s="61"/>
+      <c r="A39" s="62"/>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A40" s="61"/>
+      <c r="A40" s="62"/>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A41" s="61"/>
+      <c r="A41" s="62"/>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A42" s="61"/>
+      <c r="A42" s="62"/>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A43" s="61"/>
+      <c r="A43" s="62"/>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A44" s="61"/>
+      <c r="A44" s="62"/>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A45" s="61"/>
+      <c r="A45" s="62"/>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A46" s="61"/>
+      <c r="A46" s="62"/>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A47" s="61"/>
+      <c r="A47" s="62"/>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A48" s="61"/>
+      <c r="A48" s="62"/>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A49" s="61"/>
+      <c r="A49" s="62"/>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A50" s="61"/>
+      <c r="A50" s="62"/>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A51" s="61"/>
+      <c r="A51" s="62"/>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A52" s="61"/>
+      <c r="A52" s="62"/>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A53" s="61"/>
+      <c r="A53" s="62"/>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A54" s="61"/>
+      <c r="A54" s="62"/>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A55" s="61"/>
+      <c r="A55" s="62"/>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A56" s="61"/>
+      <c r="A56" s="62"/>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A57" s="61"/>
+      <c r="A57" s="62"/>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A58" s="61"/>
+      <c r="A58" s="62"/>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A59" s="61"/>
+      <c r="A59" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4712,6 +4720,273 @@
       <c r="C33" s="8">
         <f>1-(8/31)</f>
         <v>0.74193548387096775</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D38C5368-3EDC-40CB-9BB2-1236C3F3E0E9}">
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.6640625" style="3"/>
+    <col min="2" max="2" width="17.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="63" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="63" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="63" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="63" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="63" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="63" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="63" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="3">
+        <v>11</v>
+      </c>
+      <c r="B12" s="63" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" s="3">
+        <v>12</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" s="3">
+        <v>13</v>
+      </c>
+      <c r="B14" s="63" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="3">
+        <v>14</v>
+      </c>
+      <c r="B15" s="63" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="3">
+        <v>15</v>
+      </c>
+      <c r="B16" s="63" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="3">
+        <v>16</v>
+      </c>
+      <c r="B17" s="63" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="3">
+        <v>17</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="3">
+        <v>18</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="3">
+        <v>19</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="3">
+        <v>20</v>
+      </c>
+      <c r="B21" s="63" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="3">
+        <v>21</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="3">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="3">
+        <v>23</v>
+      </c>
+      <c r="B24" s="63" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" s="3">
+        <v>24</v>
+      </c>
+      <c r="B25" s="63" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" s="3">
+        <v>25</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" s="3">
+        <v>26</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="3">
+        <v>27</v>
+      </c>
+      <c r="B28" s="63" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="3">
+        <v>28</v>
+      </c>
+      <c r="B29" s="63" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" s="3">
+        <v>29</v>
+      </c>
+      <c r="B30" s="63"/>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" s="3">
+        <v>30</v>
+      </c>
+      <c r="B31" s="63"/>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B33" t="s">
+        <v>568</v>
+      </c>
+      <c r="C33" s="8">
+        <f>1-(9/28)</f>
+        <v>0.6785714285714286</v>
       </c>
     </row>
   </sheetData>
@@ -20195,553 +20470,497 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="52" t="s">
         <v>469</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="54" t="s">
+      <c r="B1" s="53"/>
+      <c r="C1" s="11" t="s">
         <v>470</v>
       </c>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="56"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="13"/>
     </row>
     <row r="2" spans="1:12" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="17"/>
-      <c r="B2" s="18"/>
-      <c r="C2" s="57" t="s">
+      <c r="A2" s="54"/>
+      <c r="B2" s="55"/>
+      <c r="C2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="58"/>
-      <c r="E2" s="57" t="s">
-        <v>57</v>
-      </c>
-      <c r="F2" s="58"/>
-      <c r="G2" s="57" t="s">
+      <c r="D2" s="15"/>
+      <c r="E2" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="G2" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="H2" s="58"/>
-      <c r="I2" s="59" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>481</v>
       </c>
-      <c r="J2" s="58"/>
-      <c r="K2" s="57" t="s">
+      <c r="J2" s="15"/>
+      <c r="K2" s="14" t="s">
         <v>377</v>
       </c>
-      <c r="L2" s="58"/>
+      <c r="L2" s="15"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="56" t="s">
         <v>471</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="44" t="s">
+      <c r="B3" s="57"/>
+      <c r="C3" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="45"/>
-      <c r="E3" s="46" t="s">
+      <c r="D3" s="44"/>
+      <c r="E3" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="F3" s="47"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="25"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="25"/>
-      <c r="K3" s="24"/>
-      <c r="L3" s="30"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="41"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="41"/>
+      <c r="K3" s="40"/>
+      <c r="L3" s="42"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A4" s="12"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="37"/>
-      <c r="F4" s="38"/>
-      <c r="G4" s="26"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="26"/>
-      <c r="J4" s="27"/>
-      <c r="K4" s="26"/>
-      <c r="L4" s="31"/>
+      <c r="A4" s="49"/>
+      <c r="B4" s="48"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="28"/>
+      <c r="K4" s="27"/>
+      <c r="L4" s="32"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A5" s="12"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="29"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="29"/>
-      <c r="K5" s="28"/>
-      <c r="L5" s="32"/>
+      <c r="A5" s="49"/>
+      <c r="B5" s="48"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="29"/>
+      <c r="L5" s="33"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="58" t="s">
         <v>472</v>
       </c>
-      <c r="B6" s="22"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="34"/>
-      <c r="E6" s="35" t="s">
+      <c r="B6" s="59"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="19" t="s">
         <v>482</v>
       </c>
-      <c r="F6" s="36"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="42"/>
-      <c r="I6" s="41"/>
-      <c r="J6" s="42"/>
-      <c r="K6" s="41"/>
-      <c r="L6" s="43"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="25"/>
+      <c r="J6" s="26"/>
+      <c r="K6" s="25"/>
+      <c r="L6" s="31"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A7" s="23"/>
-      <c r="B7" s="22"/>
-      <c r="C7" s="34"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="37"/>
-      <c r="F7" s="38"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="26"/>
-      <c r="J7" s="27"/>
-      <c r="K7" s="26"/>
-      <c r="L7" s="31"/>
+      <c r="A7" s="60"/>
+      <c r="B7" s="59"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="27"/>
+      <c r="J7" s="28"/>
+      <c r="K7" s="27"/>
+      <c r="L7" s="32"/>
     </row>
     <row r="8" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="23"/>
-      <c r="B8" s="22"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="29"/>
-      <c r="I8" s="28"/>
-      <c r="J8" s="29"/>
-      <c r="K8" s="28"/>
-      <c r="L8" s="32"/>
+      <c r="A8" s="60"/>
+      <c r="B8" s="59"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="29"/>
+      <c r="J8" s="30"/>
+      <c r="K8" s="29"/>
+      <c r="L8" s="33"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="47" t="s">
         <v>473</v>
       </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="33"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="41"/>
-      <c r="H9" s="42"/>
-      <c r="I9" s="41"/>
-      <c r="J9" s="42"/>
-      <c r="K9" s="41"/>
-      <c r="L9" s="43"/>
+      <c r="B9" s="48"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="25"/>
+      <c r="J9" s="26"/>
+      <c r="K9" s="25"/>
+      <c r="L9" s="31"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A10" s="12"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="37"/>
-      <c r="F10" s="38"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="27"/>
-      <c r="K10" s="26"/>
-      <c r="L10" s="31"/>
+      <c r="A10" s="49"/>
+      <c r="B10" s="48"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="28"/>
+      <c r="K10" s="27"/>
+      <c r="L10" s="32"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A11" s="12"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="34"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="39"/>
-      <c r="F11" s="40"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="29"/>
-      <c r="I11" s="28"/>
-      <c r="J11" s="29"/>
-      <c r="K11" s="28"/>
-      <c r="L11" s="32"/>
+      <c r="A11" s="49"/>
+      <c r="B11" s="48"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="29"/>
+      <c r="J11" s="30"/>
+      <c r="K11" s="29"/>
+      <c r="L11" s="33"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="47" t="s">
         <v>474</v>
       </c>
-      <c r="B12" s="11"/>
-      <c r="C12" s="33"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="35"/>
-      <c r="F12" s="36"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
-      <c r="I12" s="41"/>
-      <c r="J12" s="42"/>
-      <c r="K12" s="41"/>
-      <c r="L12" s="43"/>
+      <c r="B12" s="48"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="25"/>
+      <c r="J12" s="26"/>
+      <c r="K12" s="25"/>
+      <c r="L12" s="31"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A13" s="12"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="38"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="27"/>
-      <c r="I13" s="26"/>
-      <c r="J13" s="27"/>
-      <c r="K13" s="26"/>
-      <c r="L13" s="31"/>
+      <c r="A13" s="49"/>
+      <c r="B13" s="48"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="28"/>
+      <c r="K13" s="27"/>
+      <c r="L13" s="32"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A14" s="12"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="34"/>
-      <c r="D14" s="34"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="40"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="29"/>
-      <c r="I14" s="28"/>
-      <c r="J14" s="29"/>
-      <c r="K14" s="28"/>
-      <c r="L14" s="32"/>
+      <c r="A14" s="49"/>
+      <c r="B14" s="48"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="29"/>
+      <c r="J14" s="30"/>
+      <c r="K14" s="29"/>
+      <c r="L14" s="33"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="47" t="s">
         <v>475</v>
       </c>
-      <c r="B15" s="11"/>
-      <c r="C15" s="33"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="36"/>
-      <c r="G15" s="41"/>
-      <c r="H15" s="42"/>
-      <c r="I15" s="41"/>
-      <c r="J15" s="42"/>
-      <c r="K15" s="41"/>
-      <c r="L15" s="43"/>
+      <c r="B15" s="48"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="26"/>
+      <c r="I15" s="25"/>
+      <c r="J15" s="26"/>
+      <c r="K15" s="25"/>
+      <c r="L15" s="31"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A16" s="12"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="37"/>
-      <c r="F16" s="38"/>
-      <c r="G16" s="26"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="26"/>
-      <c r="J16" s="27"/>
-      <c r="K16" s="26"/>
-      <c r="L16" s="31"/>
+      <c r="A16" s="49"/>
+      <c r="B16" s="48"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="27"/>
+      <c r="J16" s="28"/>
+      <c r="K16" s="27"/>
+      <c r="L16" s="32"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A17" s="12"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="34"/>
-      <c r="D17" s="34"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="40"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="29"/>
-      <c r="I17" s="28"/>
-      <c r="J17" s="29"/>
-      <c r="K17" s="28"/>
-      <c r="L17" s="32"/>
+      <c r="A17" s="49"/>
+      <c r="B17" s="48"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="29"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="29"/>
+      <c r="J17" s="30"/>
+      <c r="K17" s="29"/>
+      <c r="L17" s="33"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="47" t="s">
         <v>476</v>
       </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="33"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="35"/>
-      <c r="F18" s="36"/>
-      <c r="G18" s="41"/>
-      <c r="H18" s="42"/>
-      <c r="I18" s="41"/>
-      <c r="J18" s="42"/>
-      <c r="K18" s="41"/>
-      <c r="L18" s="43"/>
+      <c r="B18" s="48"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="20"/>
+      <c r="G18" s="25"/>
+      <c r="H18" s="26"/>
+      <c r="I18" s="25"/>
+      <c r="J18" s="26"/>
+      <c r="K18" s="25"/>
+      <c r="L18" s="31"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A19" s="12"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="38"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="27"/>
-      <c r="I19" s="26"/>
-      <c r="J19" s="27"/>
-      <c r="K19" s="26"/>
-      <c r="L19" s="31"/>
+      <c r="A19" s="49"/>
+      <c r="B19" s="48"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="28"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="28"/>
+      <c r="K19" s="27"/>
+      <c r="L19" s="32"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A20" s="12"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="34"/>
-      <c r="D20" s="34"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="40"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="29"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="29"/>
-      <c r="K20" s="28"/>
-      <c r="L20" s="32"/>
+      <c r="A20" s="49"/>
+      <c r="B20" s="48"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="30"/>
+      <c r="I20" s="29"/>
+      <c r="J20" s="30"/>
+      <c r="K20" s="29"/>
+      <c r="L20" s="33"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="47" t="s">
         <v>477</v>
       </c>
-      <c r="B21" s="11"/>
-      <c r="C21" s="33"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="35"/>
-      <c r="F21" s="36"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="42"/>
-      <c r="I21" s="41"/>
-      <c r="J21" s="42"/>
-      <c r="K21" s="41"/>
-      <c r="L21" s="43"/>
+      <c r="B21" s="48"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="25"/>
+      <c r="H21" s="26"/>
+      <c r="I21" s="25"/>
+      <c r="J21" s="26"/>
+      <c r="K21" s="25"/>
+      <c r="L21" s="31"/>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A22" s="12"/>
-      <c r="B22" s="11"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="37"/>
-      <c r="F22" s="38"/>
-      <c r="G22" s="26"/>
-      <c r="H22" s="27"/>
-      <c r="I22" s="26"/>
-      <c r="J22" s="27"/>
-      <c r="K22" s="26"/>
-      <c r="L22" s="31"/>
+      <c r="A22" s="49"/>
+      <c r="B22" s="48"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="28"/>
+      <c r="I22" s="27"/>
+      <c r="J22" s="28"/>
+      <c r="K22" s="27"/>
+      <c r="L22" s="32"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A23" s="12"/>
-      <c r="B23" s="11"/>
-      <c r="C23" s="34"/>
-      <c r="D23" s="34"/>
-      <c r="E23" s="39"/>
-      <c r="F23" s="40"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="29"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="29"/>
-      <c r="K23" s="28"/>
-      <c r="L23" s="32"/>
+      <c r="A23" s="49"/>
+      <c r="B23" s="48"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="30"/>
+      <c r="I23" s="29"/>
+      <c r="J23" s="30"/>
+      <c r="K23" s="29"/>
+      <c r="L23" s="33"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="47" t="s">
         <v>478</v>
       </c>
-      <c r="B24" s="11"/>
-      <c r="C24" s="33"/>
-      <c r="D24" s="34"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="41"/>
-      <c r="H24" s="42"/>
-      <c r="I24" s="41"/>
-      <c r="J24" s="42"/>
-      <c r="K24" s="41"/>
-      <c r="L24" s="43"/>
+      <c r="B24" s="48"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="25"/>
+      <c r="H24" s="26"/>
+      <c r="I24" s="25"/>
+      <c r="J24" s="26"/>
+      <c r="K24" s="25"/>
+      <c r="L24" s="31"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A25" s="12"/>
-      <c r="B25" s="11"/>
-      <c r="C25" s="34"/>
-      <c r="D25" s="34"/>
-      <c r="E25" s="37"/>
-      <c r="F25" s="38"/>
-      <c r="G25" s="26"/>
-      <c r="H25" s="27"/>
-      <c r="I25" s="26"/>
-      <c r="J25" s="27"/>
-      <c r="K25" s="26"/>
-      <c r="L25" s="31"/>
+      <c r="A25" s="49"/>
+      <c r="B25" s="48"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="28"/>
+      <c r="I25" s="27"/>
+      <c r="J25" s="28"/>
+      <c r="K25" s="27"/>
+      <c r="L25" s="32"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A26" s="12"/>
-      <c r="B26" s="11"/>
-      <c r="C26" s="34"/>
-      <c r="D26" s="34"/>
-      <c r="E26" s="39"/>
-      <c r="F26" s="40"/>
-      <c r="G26" s="28"/>
-      <c r="H26" s="29"/>
-      <c r="I26" s="28"/>
-      <c r="J26" s="29"/>
-      <c r="K26" s="28"/>
-      <c r="L26" s="32"/>
+      <c r="A26" s="49"/>
+      <c r="B26" s="48"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="29"/>
+      <c r="H26" s="30"/>
+      <c r="I26" s="29"/>
+      <c r="J26" s="30"/>
+      <c r="K26" s="29"/>
+      <c r="L26" s="33"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A27" s="10" t="s">
+      <c r="A27" s="47" t="s">
         <v>479</v>
       </c>
-      <c r="B27" s="11"/>
-      <c r="C27" s="33"/>
-      <c r="D27" s="34"/>
-      <c r="E27" s="35"/>
-      <c r="F27" s="36"/>
-      <c r="G27" s="41"/>
-      <c r="H27" s="42"/>
-      <c r="I27" s="41"/>
-      <c r="J27" s="42"/>
-      <c r="K27" s="41"/>
-      <c r="L27" s="43"/>
+      <c r="B27" s="48"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="25"/>
+      <c r="H27" s="26"/>
+      <c r="I27" s="25"/>
+      <c r="J27" s="26"/>
+      <c r="K27" s="25"/>
+      <c r="L27" s="31"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A28" s="12"/>
-      <c r="B28" s="11"/>
-      <c r="C28" s="34"/>
-      <c r="D28" s="34"/>
-      <c r="E28" s="37"/>
-      <c r="F28" s="38"/>
-      <c r="G28" s="26"/>
-      <c r="H28" s="27"/>
-      <c r="I28" s="26"/>
-      <c r="J28" s="27"/>
-      <c r="K28" s="26"/>
-      <c r="L28" s="31"/>
+      <c r="A28" s="49"/>
+      <c r="B28" s="48"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="22"/>
+      <c r="G28" s="27"/>
+      <c r="H28" s="28"/>
+      <c r="I28" s="27"/>
+      <c r="J28" s="28"/>
+      <c r="K28" s="27"/>
+      <c r="L28" s="32"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A29" s="12"/>
-      <c r="B29" s="11"/>
-      <c r="C29" s="34"/>
-      <c r="D29" s="34"/>
-      <c r="E29" s="39"/>
-      <c r="F29" s="40"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="29"/>
-      <c r="I29" s="28"/>
-      <c r="J29" s="29"/>
-      <c r="K29" s="28"/>
-      <c r="L29" s="32"/>
+      <c r="A29" s="49"/>
+      <c r="B29" s="48"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="24"/>
+      <c r="G29" s="29"/>
+      <c r="H29" s="30"/>
+      <c r="I29" s="29"/>
+      <c r="J29" s="30"/>
+      <c r="K29" s="29"/>
+      <c r="L29" s="33"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A30" s="10" t="s">
+      <c r="A30" s="47" t="s">
         <v>480</v>
       </c>
-      <c r="B30" s="11"/>
-      <c r="C30" s="33" t="s">
+      <c r="B30" s="48"/>
+      <c r="C30" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="D30" s="34"/>
-      <c r="E30" s="35"/>
-      <c r="F30" s="36"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="42"/>
-      <c r="I30" s="41"/>
-      <c r="J30" s="42"/>
-      <c r="K30" s="41"/>
-      <c r="L30" s="43"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="25"/>
+      <c r="J30" s="26"/>
+      <c r="K30" s="25"/>
+      <c r="L30" s="31"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A31" s="12"/>
-      <c r="B31" s="11"/>
-      <c r="C31" s="34"/>
-      <c r="D31" s="34"/>
-      <c r="E31" s="37"/>
-      <c r="F31" s="38"/>
-      <c r="G31" s="26"/>
-      <c r="H31" s="27"/>
-      <c r="I31" s="26"/>
-      <c r="J31" s="27"/>
-      <c r="K31" s="26"/>
-      <c r="L31" s="31"/>
+      <c r="A31" s="49"/>
+      <c r="B31" s="48"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="18"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="27"/>
+      <c r="H31" s="28"/>
+      <c r="I31" s="27"/>
+      <c r="J31" s="28"/>
+      <c r="K31" s="27"/>
+      <c r="L31" s="32"/>
     </row>
     <row r="32" spans="1:12" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="13"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="48"/>
-      <c r="D32" s="48"/>
-      <c r="E32" s="49"/>
-      <c r="F32" s="50"/>
-      <c r="G32" s="51"/>
-      <c r="H32" s="52"/>
-      <c r="I32" s="51"/>
-      <c r="J32" s="52"/>
-      <c r="K32" s="51"/>
-      <c r="L32" s="53"/>
+      <c r="A32" s="50"/>
+      <c r="B32" s="51"/>
+      <c r="C32" s="34"/>
+      <c r="D32" s="34"/>
+      <c r="E32" s="35"/>
+      <c r="F32" s="36"/>
+      <c r="G32" s="37"/>
+      <c r="H32" s="38"/>
+      <c r="I32" s="37"/>
+      <c r="J32" s="38"/>
+      <c r="K32" s="37"/>
+      <c r="L32" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="67">
-    <mergeCell ref="C1:L1"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="C27:D29"/>
-    <mergeCell ref="E27:F29"/>
-    <mergeCell ref="G27:H29"/>
-    <mergeCell ref="I27:J29"/>
-    <mergeCell ref="K27:L29"/>
-    <mergeCell ref="C30:D32"/>
-    <mergeCell ref="E30:F32"/>
-    <mergeCell ref="G30:H32"/>
-    <mergeCell ref="I30:J32"/>
-    <mergeCell ref="K30:L32"/>
-    <mergeCell ref="C21:D23"/>
-    <mergeCell ref="E21:F23"/>
-    <mergeCell ref="G21:H23"/>
-    <mergeCell ref="I21:J23"/>
-    <mergeCell ref="K21:L23"/>
-    <mergeCell ref="C24:D26"/>
-    <mergeCell ref="E24:F26"/>
-    <mergeCell ref="G24:H26"/>
-    <mergeCell ref="I24:J26"/>
-    <mergeCell ref="K24:L26"/>
-    <mergeCell ref="C15:D17"/>
-    <mergeCell ref="E15:F17"/>
-    <mergeCell ref="G15:H17"/>
-    <mergeCell ref="I15:J17"/>
-    <mergeCell ref="K15:L17"/>
-    <mergeCell ref="C18:D20"/>
-    <mergeCell ref="E18:F20"/>
-    <mergeCell ref="G18:H20"/>
-    <mergeCell ref="I18:J20"/>
-    <mergeCell ref="K18:L20"/>
-    <mergeCell ref="E9:F11"/>
-    <mergeCell ref="G9:H11"/>
-    <mergeCell ref="I9:J11"/>
-    <mergeCell ref="K9:L11"/>
-    <mergeCell ref="C12:D14"/>
-    <mergeCell ref="E12:F14"/>
-    <mergeCell ref="G12:H14"/>
-    <mergeCell ref="I12:J14"/>
-    <mergeCell ref="K12:L14"/>
-    <mergeCell ref="C9:D11"/>
-    <mergeCell ref="I3:J5"/>
-    <mergeCell ref="K3:L5"/>
-    <mergeCell ref="C6:D8"/>
-    <mergeCell ref="E6:F8"/>
-    <mergeCell ref="G6:H8"/>
-    <mergeCell ref="I6:J8"/>
-    <mergeCell ref="K6:L8"/>
-    <mergeCell ref="C3:D5"/>
-    <mergeCell ref="E3:F5"/>
-    <mergeCell ref="G3:H5"/>
     <mergeCell ref="A30:B32"/>
     <mergeCell ref="A1:B2"/>
     <mergeCell ref="A3:B5"/>
@@ -20753,6 +20972,62 @@
     <mergeCell ref="A21:B23"/>
     <mergeCell ref="A24:B26"/>
     <mergeCell ref="A27:B29"/>
+    <mergeCell ref="I3:J5"/>
+    <mergeCell ref="K3:L5"/>
+    <mergeCell ref="C6:D8"/>
+    <mergeCell ref="E6:F8"/>
+    <mergeCell ref="G6:H8"/>
+    <mergeCell ref="I6:J8"/>
+    <mergeCell ref="K6:L8"/>
+    <mergeCell ref="C3:D5"/>
+    <mergeCell ref="E3:F5"/>
+    <mergeCell ref="G3:H5"/>
+    <mergeCell ref="E9:F11"/>
+    <mergeCell ref="G9:H11"/>
+    <mergeCell ref="I9:J11"/>
+    <mergeCell ref="K9:L11"/>
+    <mergeCell ref="C12:D14"/>
+    <mergeCell ref="E12:F14"/>
+    <mergeCell ref="G12:H14"/>
+    <mergeCell ref="I12:J14"/>
+    <mergeCell ref="K12:L14"/>
+    <mergeCell ref="C9:D11"/>
+    <mergeCell ref="C18:D20"/>
+    <mergeCell ref="E18:F20"/>
+    <mergeCell ref="G18:H20"/>
+    <mergeCell ref="I18:J20"/>
+    <mergeCell ref="K18:L20"/>
+    <mergeCell ref="C15:D17"/>
+    <mergeCell ref="E15:F17"/>
+    <mergeCell ref="G15:H17"/>
+    <mergeCell ref="I15:J17"/>
+    <mergeCell ref="K15:L17"/>
+    <mergeCell ref="C24:D26"/>
+    <mergeCell ref="E24:F26"/>
+    <mergeCell ref="G24:H26"/>
+    <mergeCell ref="I24:J26"/>
+    <mergeCell ref="K24:L26"/>
+    <mergeCell ref="C21:D23"/>
+    <mergeCell ref="E21:F23"/>
+    <mergeCell ref="G21:H23"/>
+    <mergeCell ref="I21:J23"/>
+    <mergeCell ref="K21:L23"/>
+    <mergeCell ref="C30:D32"/>
+    <mergeCell ref="E30:F32"/>
+    <mergeCell ref="G30:H32"/>
+    <mergeCell ref="I30:J32"/>
+    <mergeCell ref="K30:L32"/>
+    <mergeCell ref="C27:D29"/>
+    <mergeCell ref="E27:F29"/>
+    <mergeCell ref="G27:H29"/>
+    <mergeCell ref="I27:J29"/>
+    <mergeCell ref="K27:L29"/>
+    <mergeCell ref="C1:L1"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="K2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Chapter 8 Project Cost Management
</commit_message>
<xml_diff>
--- a/PMBOK_ITTOs_Interactive_Dashboard_2025-09-12.xlsx
+++ b/PMBOK_ITTOs_Interactive_Dashboard_2025-09-12.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eric.hayes\Documents\PMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1167CD95-E36E-4031-8FAA-0F7BE55DBAFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F0368C-0660-4D91-8A9A-A75EE3B5CBAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-11235" yWindow="-16395" windowWidth="29040" windowHeight="16440" firstSheet="10" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="16220" firstSheet="14" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Definitions" sheetId="16" r:id="rId1"/>
@@ -29,6 +29,7 @@
     <sheet name="CH5 IntegrationMGMT" sheetId="11" r:id="rId14"/>
     <sheet name="CH6 Project Scope Management" sheetId="15" r:id="rId15"/>
     <sheet name="CH7 Project Schedule Management" sheetId="17" r:id="rId16"/>
+    <sheet name="CH8 Project Cost Management" sheetId="18" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="Slicer_ITTO_Name">#N/A</definedName>
@@ -42,9 +43,9 @@
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{46BE6895-7355-4a93-B00E-2C351335B9C9}">
       <x15:slicerCaches xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
-        <x14:slicerCache r:id="rId17"/>
         <x14:slicerCache r:id="rId18"/>
         <x14:slicerCache r:id="rId19"/>
+        <x14:slicerCache r:id="rId20"/>
       </x15:slicerCaches>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -63,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6153" uniqueCount="571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6183" uniqueCount="571">
   <si>
     <t>Process</t>
   </si>
@@ -2414,7 +2415,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2436,114 +2437,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2586,13 +2480,121 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2623,7 +2625,7 @@
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>104775</xdr:colOff>
-      <xdr:row>700</xdr:row>
+      <xdr:row>701</xdr:row>
       <xdr:rowOff>142875</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
@@ -2701,7 +2703,7 @@
     <xdr:to>
       <xdr:col>13</xdr:col>
       <xdr:colOff>666750</xdr:colOff>
-      <xdr:row>147</xdr:row>
+      <xdr:row>177</xdr:row>
       <xdr:rowOff>114301</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
@@ -2773,13 +2775,13 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>152400</xdr:colOff>
-      <xdr:row>147</xdr:row>
+      <xdr:row>177</xdr:row>
       <xdr:rowOff>161925</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
       <xdr:colOff>95250</xdr:colOff>
-      <xdr:row>700</xdr:row>
+      <xdr:row>701</xdr:row>
       <xdr:rowOff>9525</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
@@ -2893,12 +2895,12 @@
   <autoFilter ref="A1:G671" xr:uid="{4601F446-1501-4E3F-8747-71EE2C76E6AC}">
     <filterColumn colId="0">
       <filters>
-        <filter val="Develop Schedule"/>
+        <filter val="Determine Budget"/>
       </filters>
     </filterColumn>
     <filterColumn colId="3">
       <filters>
-        <filter val="Output"/>
+        <filter val="Input"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -3273,183 +3275,183 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="62" t="s">
         <v>483</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A2" s="62"/>
+      <c r="A2" s="63"/>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A3" s="62"/>
+      <c r="A3" s="63"/>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" s="62"/>
+      <c r="A4" s="63"/>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A5" s="62"/>
+      <c r="A5" s="63"/>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A6" s="62"/>
+      <c r="A6" s="63"/>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A7" s="62"/>
+      <c r="A7" s="63"/>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A8" s="62"/>
+      <c r="A8" s="63"/>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A9" s="62"/>
+      <c r="A9" s="63"/>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A10" s="62"/>
+      <c r="A10" s="63"/>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A11" s="62"/>
+      <c r="A11" s="63"/>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A12" s="62"/>
+      <c r="A12" s="63"/>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A13" s="62"/>
+      <c r="A13" s="63"/>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A14" s="62"/>
+      <c r="A14" s="63"/>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A15" s="62"/>
+      <c r="A15" s="63"/>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A16" s="62"/>
+      <c r="A16" s="63"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" s="62"/>
+      <c r="A17" s="63"/>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A18" s="62"/>
+      <c r="A18" s="63"/>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A19" s="62"/>
+      <c r="A19" s="63"/>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A20" s="62"/>
+      <c r="A20" s="63"/>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A21" s="62"/>
+      <c r="A21" s="63"/>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A22" s="62"/>
+      <c r="A22" s="63"/>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A23" s="62"/>
+      <c r="A23" s="63"/>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" s="62"/>
+      <c r="A24" s="63"/>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" s="62"/>
+      <c r="A25" s="63"/>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A26" s="62"/>
+      <c r="A26" s="63"/>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" s="62"/>
+      <c r="A27" s="63"/>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A28" s="62"/>
+      <c r="A28" s="63"/>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A29" s="62"/>
+      <c r="A29" s="63"/>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A30" s="62"/>
+      <c r="A30" s="63"/>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A31" s="62"/>
+      <c r="A31" s="63"/>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A32" s="62"/>
+      <c r="A32" s="63"/>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" s="62"/>
+      <c r="A33" s="63"/>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A34" s="62"/>
+      <c r="A34" s="63"/>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A35" s="62"/>
+      <c r="A35" s="63"/>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A36" s="62"/>
+      <c r="A36" s="63"/>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A37" s="62"/>
+      <c r="A37" s="63"/>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A38" s="62"/>
+      <c r="A38" s="63"/>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A39" s="62"/>
+      <c r="A39" s="63"/>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A40" s="62"/>
+      <c r="A40" s="63"/>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A41" s="62"/>
+      <c r="A41" s="63"/>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A42" s="62"/>
+      <c r="A42" s="63"/>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A43" s="62"/>
+      <c r="A43" s="63"/>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A44" s="62"/>
+      <c r="A44" s="63"/>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A45" s="62"/>
+      <c r="A45" s="63"/>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A46" s="62"/>
+      <c r="A46" s="63"/>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A47" s="62"/>
+      <c r="A47" s="63"/>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A48" s="62"/>
+      <c r="A48" s="63"/>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A49" s="62"/>
+      <c r="A49" s="63"/>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A50" s="62"/>
+      <c r="A50" s="63"/>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A51" s="62"/>
+      <c r="A51" s="63"/>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A52" s="62"/>
+      <c r="A52" s="63"/>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A53" s="62"/>
+      <c r="A53" s="63"/>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A54" s="62"/>
+      <c r="A54" s="63"/>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A55" s="62"/>
+      <c r="A55" s="63"/>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A56" s="62"/>
+      <c r="A56" s="63"/>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A57" s="62"/>
+      <c r="A57" s="63"/>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A58" s="62"/>
+      <c r="A58" s="63"/>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A59" s="62"/>
+      <c r="A59" s="63"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4772,7 +4774,7 @@
       <c r="A5" s="3">
         <v>4</v>
       </c>
-      <c r="B5" s="63" t="s">
+      <c r="B5" s="11" t="s">
         <v>487</v>
       </c>
     </row>
@@ -4780,7 +4782,7 @@
       <c r="A6" s="3">
         <v>5</v>
       </c>
-      <c r="B6" s="63" t="s">
+      <c r="B6" s="11" t="s">
         <v>488</v>
       </c>
     </row>
@@ -4788,7 +4790,7 @@
       <c r="A7" s="3">
         <v>6</v>
       </c>
-      <c r="B7" s="63" t="s">
+      <c r="B7" s="11" t="s">
         <v>488</v>
       </c>
     </row>
@@ -4796,7 +4798,7 @@
       <c r="A8" s="3">
         <v>7</v>
       </c>
-      <c r="B8" s="63" t="s">
+      <c r="B8" s="11" t="s">
         <v>487</v>
       </c>
     </row>
@@ -4804,7 +4806,7 @@
       <c r="A9" s="3">
         <v>8</v>
       </c>
-      <c r="B9" s="63" t="s">
+      <c r="B9" s="11" t="s">
         <v>488</v>
       </c>
     </row>
@@ -4812,7 +4814,7 @@
       <c r="A10" s="3">
         <v>9</v>
       </c>
-      <c r="B10" s="63" t="s">
+      <c r="B10" s="11" t="s">
         <v>488</v>
       </c>
     </row>
@@ -4820,7 +4822,7 @@
       <c r="A11" s="3">
         <v>10</v>
       </c>
-      <c r="B11" s="63" t="s">
+      <c r="B11" s="11" t="s">
         <v>489</v>
       </c>
     </row>
@@ -4828,7 +4830,7 @@
       <c r="A12" s="3">
         <v>11</v>
       </c>
-      <c r="B12" s="63" t="s">
+      <c r="B12" s="11" t="s">
         <v>489</v>
       </c>
     </row>
@@ -4844,7 +4846,7 @@
       <c r="A14" s="3">
         <v>13</v>
       </c>
-      <c r="B14" s="63" t="s">
+      <c r="B14" s="11" t="s">
         <v>488</v>
       </c>
     </row>
@@ -4852,7 +4854,7 @@
       <c r="A15" s="3">
         <v>14</v>
       </c>
-      <c r="B15" s="63" t="s">
+      <c r="B15" s="11" t="s">
         <v>486</v>
       </c>
     </row>
@@ -4860,7 +4862,7 @@
       <c r="A16" s="3">
         <v>15</v>
       </c>
-      <c r="B16" s="63" t="s">
+      <c r="B16" s="11" t="s">
         <v>489</v>
       </c>
     </row>
@@ -4868,7 +4870,7 @@
       <c r="A17" s="3">
         <v>16</v>
       </c>
-      <c r="B17" s="63" t="s">
+      <c r="B17" s="11" t="s">
         <v>487</v>
       </c>
     </row>
@@ -4900,7 +4902,7 @@
       <c r="A21" s="3">
         <v>20</v>
       </c>
-      <c r="B21" s="63" t="s">
+      <c r="B21" s="11" t="s">
         <v>489</v>
       </c>
     </row>
@@ -4924,7 +4926,7 @@
       <c r="A24" s="3">
         <v>23</v>
       </c>
-      <c r="B24" s="63" t="s">
+      <c r="B24" s="11" t="s">
         <v>489</v>
       </c>
     </row>
@@ -4932,7 +4934,7 @@
       <c r="A25" s="3">
         <v>24</v>
       </c>
-      <c r="B25" s="63" t="s">
+      <c r="B25" s="11" t="s">
         <v>487</v>
       </c>
     </row>
@@ -4956,7 +4958,7 @@
       <c r="A28" s="3">
         <v>27</v>
       </c>
-      <c r="B28" s="63" t="s">
+      <c r="B28" s="11" t="s">
         <v>486</v>
       </c>
     </row>
@@ -4964,7 +4966,7 @@
       <c r="A29" s="3">
         <v>28</v>
       </c>
-      <c r="B29" s="63" t="s">
+      <c r="B29" s="11" t="s">
         <v>488</v>
       </c>
     </row>
@@ -4972,13 +4974,13 @@
       <c r="A30" s="3">
         <v>29</v>
       </c>
-      <c r="B30" s="63"/>
+      <c r="B30" s="11"/>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
         <v>30</v>
       </c>
-      <c r="B31" s="63"/>
+      <c r="B31" s="11"/>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B33" t="s">
@@ -4987,6 +4989,271 @@
       <c r="C33" s="8">
         <f>1-(9/28)</f>
         <v>0.6785714285714286</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3398292A-1345-42A0-987A-80BEB89E4B07}">
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.6640625" style="3"/>
+    <col min="2" max="2" width="17.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="64" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="64" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="64" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="64" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="64" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="64" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="64" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="64" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="3">
+        <v>11</v>
+      </c>
+      <c r="B12" s="64" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" s="3">
+        <v>12</v>
+      </c>
+      <c r="B13" s="64" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" s="3">
+        <v>13</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="3">
+        <v>14</v>
+      </c>
+      <c r="B15" s="64" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="3">
+        <v>15</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="3">
+        <v>16</v>
+      </c>
+      <c r="B17" s="64" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="3">
+        <v>17</v>
+      </c>
+      <c r="B18" s="64" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="3">
+        <v>18</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="3">
+        <v>19</v>
+      </c>
+      <c r="B20" s="64" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="3">
+        <v>20</v>
+      </c>
+      <c r="B21" s="64" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="3">
+        <v>21</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="3">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="3">
+        <v>23</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" s="3">
+        <v>24</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" s="3">
+        <v>25</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" s="3">
+        <v>26</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="3">
+        <v>27</v>
+      </c>
+      <c r="B28" s="64" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="3">
+        <v>28</v>
+      </c>
+      <c r="B29" s="64"/>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" s="3">
+        <v>29</v>
+      </c>
+      <c r="B30" s="64"/>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" s="3">
+        <v>30</v>
+      </c>
+      <c r="B31" s="64"/>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B33" t="s">
+        <v>568</v>
+      </c>
+      <c r="C33" s="8">
+        <f>1-(9/27)</f>
+        <v>0.66666666666666674</v>
       </c>
     </row>
   </sheetData>
@@ -8274,7 +8541,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>125</v>
       </c>
@@ -8297,7 +8564,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>125</v>
       </c>
@@ -8320,7 +8587,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>125</v>
       </c>
@@ -8343,7 +8610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>125</v>
       </c>
@@ -8366,7 +8633,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>125</v>
       </c>
@@ -8389,7 +8656,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>125</v>
       </c>
@@ -8412,7 +8679,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>125</v>
       </c>
@@ -8964,7 +9231,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="173" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>151</v>
       </c>
@@ -8987,7 +9254,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="174" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>151</v>
       </c>
@@ -9010,7 +9277,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="175" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>151</v>
       </c>
@@ -9033,7 +9300,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="176" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>151</v>
       </c>
@@ -9056,7 +9323,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="177" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>151</v>
       </c>
@@ -9079,7 +9346,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="178" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>151</v>
       </c>
@@ -20470,497 +20737,553 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="17" t="s">
         <v>469</v>
       </c>
-      <c r="B1" s="53"/>
-      <c r="C1" s="11" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="56" t="s">
         <v>470</v>
       </c>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="13"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="58"/>
     </row>
     <row r="2" spans="1:12" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="54"/>
-      <c r="B2" s="55"/>
-      <c r="C2" s="14" t="s">
+      <c r="A2" s="19"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="59" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="15"/>
-      <c r="E2" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="F2" s="15"/>
-      <c r="G2" s="14" t="s">
+      <c r="D2" s="60"/>
+      <c r="E2" s="59" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="60"/>
+      <c r="G2" s="59" t="s">
         <v>249</v>
       </c>
-      <c r="H2" s="15"/>
-      <c r="I2" s="16" t="s">
+      <c r="H2" s="60"/>
+      <c r="I2" s="61" t="s">
         <v>481</v>
       </c>
-      <c r="J2" s="15"/>
-      <c r="K2" s="14" t="s">
+      <c r="J2" s="60"/>
+      <c r="K2" s="59" t="s">
         <v>377</v>
       </c>
-      <c r="L2" s="15"/>
+      <c r="L2" s="60"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="21" t="s">
         <v>471</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="43" t="s">
+      <c r="B3" s="22"/>
+      <c r="C3" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="44"/>
-      <c r="E3" s="45" t="s">
+      <c r="D3" s="47"/>
+      <c r="E3" s="48" t="s">
         <v>56</v>
       </c>
-      <c r="F3" s="46"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="40"/>
-      <c r="J3" s="41"/>
-      <c r="K3" s="40"/>
-      <c r="L3" s="42"/>
+      <c r="F3" s="49"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="27"/>
+      <c r="I3" s="26"/>
+      <c r="J3" s="27"/>
+      <c r="K3" s="26"/>
+      <c r="L3" s="32"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A4" s="49"/>
-      <c r="B4" s="48"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="27"/>
-      <c r="J4" s="28"/>
-      <c r="K4" s="27"/>
-      <c r="L4" s="32"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="39"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="29"/>
+      <c r="I4" s="28"/>
+      <c r="J4" s="29"/>
+      <c r="K4" s="28"/>
+      <c r="L4" s="33"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A5" s="49"/>
-      <c r="B5" s="48"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="29"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="29"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="29"/>
-      <c r="L5" s="33"/>
+      <c r="A5" s="14"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="30"/>
+      <c r="L5" s="34"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A6" s="58" t="s">
+      <c r="A6" s="23" t="s">
         <v>472</v>
       </c>
-      <c r="B6" s="59"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="19" t="s">
+      <c r="B6" s="24"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="36"/>
+      <c r="E6" s="37" t="s">
         <v>482</v>
       </c>
-      <c r="F6" s="20"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="25"/>
-      <c r="J6" s="26"/>
-      <c r="K6" s="25"/>
-      <c r="L6" s="31"/>
+      <c r="F6" s="38"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="44"/>
+      <c r="I6" s="43"/>
+      <c r="J6" s="44"/>
+      <c r="K6" s="43"/>
+      <c r="L6" s="45"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A7" s="60"/>
-      <c r="B7" s="59"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="28"/>
-      <c r="I7" s="27"/>
-      <c r="J7" s="28"/>
-      <c r="K7" s="27"/>
-      <c r="L7" s="32"/>
+      <c r="A7" s="25"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="40"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="29"/>
+      <c r="I7" s="28"/>
+      <c r="J7" s="29"/>
+      <c r="K7" s="28"/>
+      <c r="L7" s="33"/>
     </row>
     <row r="8" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="60"/>
-      <c r="B8" s="59"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="29"/>
-      <c r="J8" s="30"/>
-      <c r="K8" s="29"/>
-      <c r="L8" s="33"/>
+      <c r="A8" s="25"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="41"/>
+      <c r="F8" s="42"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="31"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="31"/>
+      <c r="K8" s="30"/>
+      <c r="L8" s="34"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A9" s="47" t="s">
+      <c r="A9" s="12" t="s">
         <v>473</v>
       </c>
-      <c r="B9" s="48"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="25"/>
-      <c r="J9" s="26"/>
-      <c r="K9" s="25"/>
-      <c r="L9" s="31"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="38"/>
+      <c r="G9" s="43"/>
+      <c r="H9" s="44"/>
+      <c r="I9" s="43"/>
+      <c r="J9" s="44"/>
+      <c r="K9" s="43"/>
+      <c r="L9" s="45"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A10" s="49"/>
-      <c r="B10" s="48"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="27"/>
-      <c r="J10" s="28"/>
-      <c r="K10" s="27"/>
-      <c r="L10" s="32"/>
+      <c r="A10" s="14"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="36"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="40"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="29"/>
+      <c r="K10" s="28"/>
+      <c r="L10" s="33"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A11" s="49"/>
-      <c r="B11" s="48"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="29"/>
-      <c r="H11" s="30"/>
-      <c r="I11" s="29"/>
-      <c r="J11" s="30"/>
-      <c r="K11" s="29"/>
-      <c r="L11" s="33"/>
+      <c r="A11" s="14"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="36"/>
+      <c r="D11" s="36"/>
+      <c r="E11" s="41"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="31"/>
+      <c r="I11" s="30"/>
+      <c r="J11" s="31"/>
+      <c r="K11" s="30"/>
+      <c r="L11" s="34"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A12" s="47" t="s">
+      <c r="A12" s="12" t="s">
         <v>474</v>
       </c>
-      <c r="B12" s="48"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="25"/>
-      <c r="J12" s="26"/>
-      <c r="K12" s="25"/>
-      <c r="L12" s="31"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="37"/>
+      <c r="F12" s="38"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="44"/>
+      <c r="I12" s="43"/>
+      <c r="J12" s="44"/>
+      <c r="K12" s="43"/>
+      <c r="L12" s="45"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A13" s="49"/>
-      <c r="B13" s="48"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="28"/>
-      <c r="I13" s="27"/>
-      <c r="J13" s="28"/>
-      <c r="K13" s="27"/>
-      <c r="L13" s="32"/>
+      <c r="A13" s="14"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="40"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="28"/>
+      <c r="J13" s="29"/>
+      <c r="K13" s="28"/>
+      <c r="L13" s="33"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A14" s="49"/>
-      <c r="B14" s="48"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="29"/>
-      <c r="H14" s="30"/>
-      <c r="I14" s="29"/>
-      <c r="J14" s="30"/>
-      <c r="K14" s="29"/>
-      <c r="L14" s="33"/>
+      <c r="A14" s="14"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="41"/>
+      <c r="F14" s="42"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="31"/>
+      <c r="I14" s="30"/>
+      <c r="J14" s="31"/>
+      <c r="K14" s="30"/>
+      <c r="L14" s="34"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A15" s="47" t="s">
+      <c r="A15" s="12" t="s">
         <v>475</v>
       </c>
-      <c r="B15" s="48"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="26"/>
-      <c r="I15" s="25"/>
-      <c r="J15" s="26"/>
-      <c r="K15" s="25"/>
-      <c r="L15" s="31"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="37"/>
+      <c r="F15" s="38"/>
+      <c r="G15" s="43"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="43"/>
+      <c r="J15" s="44"/>
+      <c r="K15" s="43"/>
+      <c r="L15" s="45"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A16" s="49"/>
-      <c r="B16" s="48"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="28"/>
-      <c r="I16" s="27"/>
-      <c r="J16" s="28"/>
-      <c r="K16" s="27"/>
-      <c r="L16" s="32"/>
+      <c r="A16" s="14"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="36"/>
+      <c r="D16" s="36"/>
+      <c r="E16" s="39"/>
+      <c r="F16" s="40"/>
+      <c r="G16" s="28"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="28"/>
+      <c r="J16" s="29"/>
+      <c r="K16" s="28"/>
+      <c r="L16" s="33"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A17" s="49"/>
-      <c r="B17" s="48"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="29"/>
-      <c r="H17" s="30"/>
-      <c r="I17" s="29"/>
-      <c r="J17" s="30"/>
-      <c r="K17" s="29"/>
-      <c r="L17" s="33"/>
+      <c r="A17" s="14"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="36"/>
+      <c r="D17" s="36"/>
+      <c r="E17" s="41"/>
+      <c r="F17" s="42"/>
+      <c r="G17" s="30"/>
+      <c r="H17" s="31"/>
+      <c r="I17" s="30"/>
+      <c r="J17" s="31"/>
+      <c r="K17" s="30"/>
+      <c r="L17" s="34"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A18" s="47" t="s">
+      <c r="A18" s="12" t="s">
         <v>476</v>
       </c>
-      <c r="B18" s="48"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="25"/>
-      <c r="J18" s="26"/>
-      <c r="K18" s="25"/>
-      <c r="L18" s="31"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="43"/>
+      <c r="H18" s="44"/>
+      <c r="I18" s="43"/>
+      <c r="J18" s="44"/>
+      <c r="K18" s="43"/>
+      <c r="L18" s="45"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A19" s="49"/>
-      <c r="B19" s="48"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="21"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="28"/>
-      <c r="I19" s="27"/>
-      <c r="J19" s="28"/>
-      <c r="K19" s="27"/>
-      <c r="L19" s="32"/>
+      <c r="A19" s="14"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="39"/>
+      <c r="F19" s="40"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="29"/>
+      <c r="I19" s="28"/>
+      <c r="J19" s="29"/>
+      <c r="K19" s="28"/>
+      <c r="L19" s="33"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A20" s="49"/>
-      <c r="B20" s="48"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="29"/>
-      <c r="H20" s="30"/>
-      <c r="I20" s="29"/>
-      <c r="J20" s="30"/>
-      <c r="K20" s="29"/>
-      <c r="L20" s="33"/>
+      <c r="A20" s="14"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="41"/>
+      <c r="F20" s="42"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="31"/>
+      <c r="I20" s="30"/>
+      <c r="J20" s="31"/>
+      <c r="K20" s="30"/>
+      <c r="L20" s="34"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A21" s="47" t="s">
+      <c r="A21" s="12" t="s">
         <v>477</v>
       </c>
-      <c r="B21" s="48"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="26"/>
-      <c r="I21" s="25"/>
-      <c r="J21" s="26"/>
-      <c r="K21" s="25"/>
-      <c r="L21" s="31"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="35"/>
+      <c r="D21" s="36"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="38"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="44"/>
+      <c r="I21" s="43"/>
+      <c r="J21" s="44"/>
+      <c r="K21" s="43"/>
+      <c r="L21" s="45"/>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A22" s="49"/>
-      <c r="B22" s="48"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="21"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="27"/>
-      <c r="H22" s="28"/>
-      <c r="I22" s="27"/>
-      <c r="J22" s="28"/>
-      <c r="K22" s="27"/>
-      <c r="L22" s="32"/>
+      <c r="A22" s="14"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="36"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="39"/>
+      <c r="F22" s="40"/>
+      <c r="G22" s="28"/>
+      <c r="H22" s="29"/>
+      <c r="I22" s="28"/>
+      <c r="J22" s="29"/>
+      <c r="K22" s="28"/>
+      <c r="L22" s="33"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A23" s="49"/>
-      <c r="B23" s="48"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="29"/>
-      <c r="H23" s="30"/>
-      <c r="I23" s="29"/>
-      <c r="J23" s="30"/>
-      <c r="K23" s="29"/>
-      <c r="L23" s="33"/>
+      <c r="A23" s="14"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="36"/>
+      <c r="D23" s="36"/>
+      <c r="E23" s="41"/>
+      <c r="F23" s="42"/>
+      <c r="G23" s="30"/>
+      <c r="H23" s="31"/>
+      <c r="I23" s="30"/>
+      <c r="J23" s="31"/>
+      <c r="K23" s="30"/>
+      <c r="L23" s="34"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A24" s="47" t="s">
+      <c r="A24" s="12" t="s">
         <v>478</v>
       </c>
-      <c r="B24" s="48"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="26"/>
-      <c r="I24" s="25"/>
-      <c r="J24" s="26"/>
-      <c r="K24" s="25"/>
-      <c r="L24" s="31"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="37"/>
+      <c r="F24" s="38"/>
+      <c r="G24" s="43"/>
+      <c r="H24" s="44"/>
+      <c r="I24" s="43"/>
+      <c r="J24" s="44"/>
+      <c r="K24" s="43"/>
+      <c r="L24" s="45"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A25" s="49"/>
-      <c r="B25" s="48"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="27"/>
-      <c r="H25" s="28"/>
-      <c r="I25" s="27"/>
-      <c r="J25" s="28"/>
-      <c r="K25" s="27"/>
-      <c r="L25" s="32"/>
+      <c r="A25" s="14"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="36"/>
+      <c r="D25" s="36"/>
+      <c r="E25" s="39"/>
+      <c r="F25" s="40"/>
+      <c r="G25" s="28"/>
+      <c r="H25" s="29"/>
+      <c r="I25" s="28"/>
+      <c r="J25" s="29"/>
+      <c r="K25" s="28"/>
+      <c r="L25" s="33"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A26" s="49"/>
-      <c r="B26" s="48"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="23"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="29"/>
-      <c r="H26" s="30"/>
-      <c r="I26" s="29"/>
-      <c r="J26" s="30"/>
-      <c r="K26" s="29"/>
-      <c r="L26" s="33"/>
+      <c r="A26" s="14"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="36"/>
+      <c r="D26" s="36"/>
+      <c r="E26" s="41"/>
+      <c r="F26" s="42"/>
+      <c r="G26" s="30"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="30"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="30"/>
+      <c r="L26" s="34"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A27" s="47" t="s">
+      <c r="A27" s="12" t="s">
         <v>479</v>
       </c>
-      <c r="B27" s="48"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="25"/>
-      <c r="H27" s="26"/>
-      <c r="I27" s="25"/>
-      <c r="J27" s="26"/>
-      <c r="K27" s="25"/>
-      <c r="L27" s="31"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="35"/>
+      <c r="D27" s="36"/>
+      <c r="E27" s="37"/>
+      <c r="F27" s="38"/>
+      <c r="G27" s="43"/>
+      <c r="H27" s="44"/>
+      <c r="I27" s="43"/>
+      <c r="J27" s="44"/>
+      <c r="K27" s="43"/>
+      <c r="L27" s="45"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A28" s="49"/>
-      <c r="B28" s="48"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="21"/>
-      <c r="F28" s="22"/>
-      <c r="G28" s="27"/>
-      <c r="H28" s="28"/>
-      <c r="I28" s="27"/>
-      <c r="J28" s="28"/>
-      <c r="K28" s="27"/>
-      <c r="L28" s="32"/>
+      <c r="A28" s="14"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="36"/>
+      <c r="D28" s="36"/>
+      <c r="E28" s="39"/>
+      <c r="F28" s="40"/>
+      <c r="G28" s="28"/>
+      <c r="H28" s="29"/>
+      <c r="I28" s="28"/>
+      <c r="J28" s="29"/>
+      <c r="K28" s="28"/>
+      <c r="L28" s="33"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A29" s="49"/>
-      <c r="B29" s="48"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="29"/>
-      <c r="H29" s="30"/>
-      <c r="I29" s="29"/>
-      <c r="J29" s="30"/>
-      <c r="K29" s="29"/>
-      <c r="L29" s="33"/>
+      <c r="A29" s="14"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="36"/>
+      <c r="D29" s="36"/>
+      <c r="E29" s="41"/>
+      <c r="F29" s="42"/>
+      <c r="G29" s="30"/>
+      <c r="H29" s="31"/>
+      <c r="I29" s="30"/>
+      <c r="J29" s="31"/>
+      <c r="K29" s="30"/>
+      <c r="L29" s="34"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A30" s="47" t="s">
+      <c r="A30" s="12" t="s">
         <v>480</v>
       </c>
-      <c r="B30" s="48"/>
-      <c r="C30" s="17" t="s">
+      <c r="B30" s="13"/>
+      <c r="C30" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="D30" s="18"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="25"/>
-      <c r="H30" s="26"/>
-      <c r="I30" s="25"/>
-      <c r="J30" s="26"/>
-      <c r="K30" s="25"/>
-      <c r="L30" s="31"/>
+      <c r="D30" s="36"/>
+      <c r="E30" s="37"/>
+      <c r="F30" s="38"/>
+      <c r="G30" s="43"/>
+      <c r="H30" s="44"/>
+      <c r="I30" s="43"/>
+      <c r="J30" s="44"/>
+      <c r="K30" s="43"/>
+      <c r="L30" s="45"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A31" s="49"/>
-      <c r="B31" s="48"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="21"/>
-      <c r="F31" s="22"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="28"/>
-      <c r="I31" s="27"/>
-      <c r="J31" s="28"/>
-      <c r="K31" s="27"/>
-      <c r="L31" s="32"/>
+      <c r="A31" s="14"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="36"/>
+      <c r="D31" s="36"/>
+      <c r="E31" s="39"/>
+      <c r="F31" s="40"/>
+      <c r="G31" s="28"/>
+      <c r="H31" s="29"/>
+      <c r="I31" s="28"/>
+      <c r="J31" s="29"/>
+      <c r="K31" s="28"/>
+      <c r="L31" s="33"/>
     </row>
     <row r="32" spans="1:12" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="50"/>
-      <c r="B32" s="51"/>
-      <c r="C32" s="34"/>
-      <c r="D32" s="34"/>
-      <c r="E32" s="35"/>
-      <c r="F32" s="36"/>
-      <c r="G32" s="37"/>
-      <c r="H32" s="38"/>
-      <c r="I32" s="37"/>
-      <c r="J32" s="38"/>
-      <c r="K32" s="37"/>
-      <c r="L32" s="39"/>
+      <c r="A32" s="15"/>
+      <c r="B32" s="16"/>
+      <c r="C32" s="50"/>
+      <c r="D32" s="50"/>
+      <c r="E32" s="51"/>
+      <c r="F32" s="52"/>
+      <c r="G32" s="53"/>
+      <c r="H32" s="54"/>
+      <c r="I32" s="53"/>
+      <c r="J32" s="54"/>
+      <c r="K32" s="53"/>
+      <c r="L32" s="55"/>
     </row>
   </sheetData>
   <mergeCells count="67">
+    <mergeCell ref="C1:L1"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="C27:D29"/>
+    <mergeCell ref="E27:F29"/>
+    <mergeCell ref="G27:H29"/>
+    <mergeCell ref="I27:J29"/>
+    <mergeCell ref="K27:L29"/>
+    <mergeCell ref="C30:D32"/>
+    <mergeCell ref="E30:F32"/>
+    <mergeCell ref="G30:H32"/>
+    <mergeCell ref="I30:J32"/>
+    <mergeCell ref="K30:L32"/>
+    <mergeCell ref="C21:D23"/>
+    <mergeCell ref="E21:F23"/>
+    <mergeCell ref="G21:H23"/>
+    <mergeCell ref="I21:J23"/>
+    <mergeCell ref="K21:L23"/>
+    <mergeCell ref="C24:D26"/>
+    <mergeCell ref="E24:F26"/>
+    <mergeCell ref="G24:H26"/>
+    <mergeCell ref="I24:J26"/>
+    <mergeCell ref="K24:L26"/>
+    <mergeCell ref="C15:D17"/>
+    <mergeCell ref="E15:F17"/>
+    <mergeCell ref="G15:H17"/>
+    <mergeCell ref="I15:J17"/>
+    <mergeCell ref="K15:L17"/>
+    <mergeCell ref="C18:D20"/>
+    <mergeCell ref="E18:F20"/>
+    <mergeCell ref="G18:H20"/>
+    <mergeCell ref="I18:J20"/>
+    <mergeCell ref="K18:L20"/>
+    <mergeCell ref="E9:F11"/>
+    <mergeCell ref="G9:H11"/>
+    <mergeCell ref="I9:J11"/>
+    <mergeCell ref="K9:L11"/>
+    <mergeCell ref="C12:D14"/>
+    <mergeCell ref="E12:F14"/>
+    <mergeCell ref="G12:H14"/>
+    <mergeCell ref="I12:J14"/>
+    <mergeCell ref="K12:L14"/>
+    <mergeCell ref="C9:D11"/>
+    <mergeCell ref="I3:J5"/>
+    <mergeCell ref="K3:L5"/>
+    <mergeCell ref="C6:D8"/>
+    <mergeCell ref="E6:F8"/>
+    <mergeCell ref="G6:H8"/>
+    <mergeCell ref="I6:J8"/>
+    <mergeCell ref="K6:L8"/>
+    <mergeCell ref="C3:D5"/>
+    <mergeCell ref="E3:F5"/>
+    <mergeCell ref="G3:H5"/>
     <mergeCell ref="A30:B32"/>
     <mergeCell ref="A1:B2"/>
     <mergeCell ref="A3:B5"/>
@@ -20972,62 +21295,6 @@
     <mergeCell ref="A21:B23"/>
     <mergeCell ref="A24:B26"/>
     <mergeCell ref="A27:B29"/>
-    <mergeCell ref="I3:J5"/>
-    <mergeCell ref="K3:L5"/>
-    <mergeCell ref="C6:D8"/>
-    <mergeCell ref="E6:F8"/>
-    <mergeCell ref="G6:H8"/>
-    <mergeCell ref="I6:J8"/>
-    <mergeCell ref="K6:L8"/>
-    <mergeCell ref="C3:D5"/>
-    <mergeCell ref="E3:F5"/>
-    <mergeCell ref="G3:H5"/>
-    <mergeCell ref="E9:F11"/>
-    <mergeCell ref="G9:H11"/>
-    <mergeCell ref="I9:J11"/>
-    <mergeCell ref="K9:L11"/>
-    <mergeCell ref="C12:D14"/>
-    <mergeCell ref="E12:F14"/>
-    <mergeCell ref="G12:H14"/>
-    <mergeCell ref="I12:J14"/>
-    <mergeCell ref="K12:L14"/>
-    <mergeCell ref="C9:D11"/>
-    <mergeCell ref="C18:D20"/>
-    <mergeCell ref="E18:F20"/>
-    <mergeCell ref="G18:H20"/>
-    <mergeCell ref="I18:J20"/>
-    <mergeCell ref="K18:L20"/>
-    <mergeCell ref="C15:D17"/>
-    <mergeCell ref="E15:F17"/>
-    <mergeCell ref="G15:H17"/>
-    <mergeCell ref="I15:J17"/>
-    <mergeCell ref="K15:L17"/>
-    <mergeCell ref="C24:D26"/>
-    <mergeCell ref="E24:F26"/>
-    <mergeCell ref="G24:H26"/>
-    <mergeCell ref="I24:J26"/>
-    <mergeCell ref="K24:L26"/>
-    <mergeCell ref="C21:D23"/>
-    <mergeCell ref="E21:F23"/>
-    <mergeCell ref="G21:H23"/>
-    <mergeCell ref="I21:J23"/>
-    <mergeCell ref="K21:L23"/>
-    <mergeCell ref="C30:D32"/>
-    <mergeCell ref="E30:F32"/>
-    <mergeCell ref="G30:H32"/>
-    <mergeCell ref="I30:J32"/>
-    <mergeCell ref="K30:L32"/>
-    <mergeCell ref="C27:D29"/>
-    <mergeCell ref="E27:F29"/>
-    <mergeCell ref="G27:H29"/>
-    <mergeCell ref="I27:J29"/>
-    <mergeCell ref="K27:L29"/>
-    <mergeCell ref="C1:L1"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="K2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Chapter 9 added but not completed
</commit_message>
<xml_diff>
--- a/PMBOK_ITTOs_Interactive_Dashboard_2025-09-12.xlsx
+++ b/PMBOK_ITTOs_Interactive_Dashboard_2025-09-12.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eric.hayes\Documents\PMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F0368C-0660-4D91-8A9A-A75EE3B5CBAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75B0AA18-BE0E-4734-9908-1040B39D053A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="16220" firstSheet="14" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="16220" firstSheet="16" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Definitions" sheetId="16" r:id="rId1"/>
@@ -30,6 +30,7 @@
     <sheet name="CH6 Project Scope Management" sheetId="15" r:id="rId15"/>
     <sheet name="CH7 Project Schedule Management" sheetId="17" r:id="rId16"/>
     <sheet name="CH8 Project Cost Management" sheetId="18" r:id="rId17"/>
+    <sheet name="CH9 Project Quality Management" sheetId="19" r:id="rId18"/>
   </sheets>
   <definedNames>
     <definedName name="Slicer_ITTO_Name">#N/A</definedName>
@@ -43,9 +44,9 @@
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{46BE6895-7355-4a93-B00E-2C351335B9C9}">
       <x15:slicerCaches xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
-        <x14:slicerCache r:id="rId18"/>
         <x14:slicerCache r:id="rId19"/>
         <x14:slicerCache r:id="rId20"/>
+        <x14:slicerCache r:id="rId21"/>
       </x15:slicerCaches>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -64,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6183" uniqueCount="571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6186" uniqueCount="571">
   <si>
     <t>Process</t>
   </si>
@@ -2415,7 +2416,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2438,6 +2439,114 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2480,121 +2589,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5033,7 +5033,7 @@
       <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="64" t="s">
+      <c r="B4" t="s">
         <v>487</v>
       </c>
     </row>
@@ -5041,7 +5041,7 @@
       <c r="A5" s="3">
         <v>4</v>
       </c>
-      <c r="B5" s="64" t="s">
+      <c r="B5" t="s">
         <v>486</v>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       <c r="A6" s="3">
         <v>5</v>
       </c>
-      <c r="B6" s="64" t="s">
+      <c r="B6" t="s">
         <v>489</v>
       </c>
     </row>
@@ -5057,7 +5057,7 @@
       <c r="A7" s="3">
         <v>6</v>
       </c>
-      <c r="B7" s="64" t="s">
+      <c r="B7" t="s">
         <v>488</v>
       </c>
     </row>
@@ -5065,7 +5065,7 @@
       <c r="A8" s="3">
         <v>7</v>
       </c>
-      <c r="B8" s="64" t="s">
+      <c r="B8" t="s">
         <v>486</v>
       </c>
     </row>
@@ -5073,7 +5073,7 @@
       <c r="A9" s="3">
         <v>8</v>
       </c>
-      <c r="B9" s="64" t="s">
+      <c r="B9" t="s">
         <v>489</v>
       </c>
     </row>
@@ -5081,7 +5081,7 @@
       <c r="A10" s="3">
         <v>9</v>
       </c>
-      <c r="B10" s="64" t="s">
+      <c r="B10" t="s">
         <v>489</v>
       </c>
     </row>
@@ -5089,7 +5089,7 @@
       <c r="A11" s="3">
         <v>10</v>
       </c>
-      <c r="B11" s="64" t="s">
+      <c r="B11" t="s">
         <v>486</v>
       </c>
     </row>
@@ -5097,7 +5097,7 @@
       <c r="A12" s="3">
         <v>11</v>
       </c>
-      <c r="B12" s="64" t="s">
+      <c r="B12" t="s">
         <v>488</v>
       </c>
     </row>
@@ -5105,7 +5105,7 @@
       <c r="A13" s="3">
         <v>12</v>
       </c>
-      <c r="B13" s="64" t="s">
+      <c r="B13" t="s">
         <v>487</v>
       </c>
     </row>
@@ -5121,7 +5121,7 @@
       <c r="A15" s="3">
         <v>14</v>
       </c>
-      <c r="B15" s="64" t="s">
+      <c r="B15" t="s">
         <v>487</v>
       </c>
     </row>
@@ -5137,7 +5137,7 @@
       <c r="A17" s="3">
         <v>16</v>
       </c>
-      <c r="B17" s="64" t="s">
+      <c r="B17" t="s">
         <v>489</v>
       </c>
     </row>
@@ -5145,7 +5145,7 @@
       <c r="A18" s="3">
         <v>17</v>
       </c>
-      <c r="B18" s="64" t="s">
+      <c r="B18" t="s">
         <v>487</v>
       </c>
     </row>
@@ -5161,7 +5161,7 @@
       <c r="A20" s="3">
         <v>19</v>
       </c>
-      <c r="B20" s="64" t="s">
+      <c r="B20" t="s">
         <v>488</v>
       </c>
     </row>
@@ -5169,7 +5169,7 @@
       <c r="A21" s="3">
         <v>20</v>
       </c>
-      <c r="B21" s="64" t="s">
+      <c r="B21" t="s">
         <v>486</v>
       </c>
     </row>
@@ -5225,7 +5225,7 @@
       <c r="A28" s="3">
         <v>27</v>
       </c>
-      <c r="B28" s="64" t="s">
+      <c r="B28" t="s">
         <v>489</v>
       </c>
     </row>
@@ -5233,19 +5233,227 @@
       <c r="A29" s="3">
         <v>28</v>
       </c>
-      <c r="B29" s="64"/>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
         <v>29</v>
       </c>
-      <c r="B30" s="64"/>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
         <v>30</v>
       </c>
-      <c r="B31" s="64"/>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B33" t="s">
+        <v>568</v>
+      </c>
+      <c r="C33" s="8">
+        <f>1-(9/27)</f>
+        <v>0.66666666666666674</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C59F0856-1182-4DCE-92BD-7D08EFFDFADB}">
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.6640625" style="3"/>
+    <col min="2" max="2" width="17.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="11"/>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="11"/>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="11"/>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="11"/>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="11"/>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="11"/>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="11"/>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="11"/>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="11"/>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="11"/>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="3">
+        <v>11</v>
+      </c>
+      <c r="B12" s="11"/>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" s="3">
+        <v>12</v>
+      </c>
+      <c r="B13" s="11"/>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" s="3">
+        <v>13</v>
+      </c>
+      <c r="B14" s="11"/>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="3">
+        <v>14</v>
+      </c>
+      <c r="B15" s="11"/>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="3">
+        <v>15</v>
+      </c>
+      <c r="B16" s="11"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="3">
+        <v>16</v>
+      </c>
+      <c r="B17" s="11"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="3">
+        <v>17</v>
+      </c>
+      <c r="B18" s="11"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="3">
+        <v>18</v>
+      </c>
+      <c r="B19" s="11"/>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="3">
+        <v>19</v>
+      </c>
+      <c r="B20" s="11"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="3">
+        <v>20</v>
+      </c>
+      <c r="B21" s="11"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="3">
+        <v>21</v>
+      </c>
+      <c r="B22" s="11"/>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="3">
+        <v>22</v>
+      </c>
+      <c r="B23" s="11"/>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="3">
+        <v>23</v>
+      </c>
+      <c r="B24" s="11"/>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" s="3">
+        <v>24</v>
+      </c>
+      <c r="B25" s="11"/>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" s="3">
+        <v>25</v>
+      </c>
+      <c r="B26" s="11"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" s="3">
+        <v>26</v>
+      </c>
+      <c r="B27" s="11"/>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="3">
+        <v>27</v>
+      </c>
+      <c r="B28" s="11"/>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="3">
+        <v>28</v>
+      </c>
+      <c r="B29" s="11"/>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" s="3">
+        <v>29</v>
+      </c>
+      <c r="B30" s="11"/>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" s="3">
+        <v>30</v>
+      </c>
+      <c r="B31" s="11"/>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B33" t="s">
@@ -20737,74 +20945,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="53" t="s">
         <v>469</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="56" t="s">
+      <c r="B1" s="54"/>
+      <c r="C1" s="12" t="s">
         <v>470</v>
       </c>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
-      <c r="L1" s="58"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="14"/>
     </row>
     <row r="2" spans="1:12" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="19"/>
-      <c r="B2" s="20"/>
-      <c r="C2" s="59" t="s">
+      <c r="A2" s="55"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="60"/>
-      <c r="E2" s="59" t="s">
-        <v>57</v>
-      </c>
-      <c r="F2" s="60"/>
-      <c r="G2" s="59" t="s">
+      <c r="D2" s="16"/>
+      <c r="E2" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="16"/>
+      <c r="G2" s="15" t="s">
         <v>249</v>
       </c>
-      <c r="H2" s="60"/>
-      <c r="I2" s="61" t="s">
+      <c r="H2" s="16"/>
+      <c r="I2" s="17" t="s">
         <v>481</v>
       </c>
-      <c r="J2" s="60"/>
-      <c r="K2" s="59" t="s">
+      <c r="J2" s="16"/>
+      <c r="K2" s="15" t="s">
         <v>377</v>
       </c>
-      <c r="L2" s="60"/>
+      <c r="L2" s="16"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="57" t="s">
         <v>471</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="46" t="s">
+      <c r="B3" s="58"/>
+      <c r="C3" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="47"/>
-      <c r="E3" s="48" t="s">
+      <c r="D3" s="45"/>
+      <c r="E3" s="46" t="s">
         <v>56</v>
       </c>
-      <c r="F3" s="49"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="27"/>
-      <c r="I3" s="26"/>
-      <c r="J3" s="27"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="32"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="42"/>
+      <c r="I3" s="41"/>
+      <c r="J3" s="42"/>
+      <c r="K3" s="41"/>
+      <c r="L3" s="43"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A4" s="14"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="40"/>
+      <c r="A4" s="50"/>
+      <c r="B4" s="49"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="23"/>
       <c r="G4" s="28"/>
       <c r="H4" s="29"/>
       <c r="I4" s="28"/>
@@ -20813,12 +21021,12 @@
       <c r="L4" s="33"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A5" s="14"/>
-      <c r="B5" s="13"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="41"/>
-      <c r="F5" s="42"/>
+      <c r="A5" s="50"/>
+      <c r="B5" s="49"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="25"/>
       <c r="G5" s="30"/>
       <c r="H5" s="31"/>
       <c r="I5" s="30"/>
@@ -20827,30 +21035,30 @@
       <c r="L5" s="34"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="59" t="s">
         <v>472</v>
       </c>
-      <c r="B6" s="24"/>
-      <c r="C6" s="35"/>
-      <c r="D6" s="36"/>
-      <c r="E6" s="37" t="s">
+      <c r="B6" s="60"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="20" t="s">
         <v>482</v>
       </c>
-      <c r="F6" s="38"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
-      <c r="I6" s="43"/>
-      <c r="J6" s="44"/>
-      <c r="K6" s="43"/>
-      <c r="L6" s="45"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="27"/>
+      <c r="K6" s="26"/>
+      <c r="L6" s="32"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A7" s="25"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="40"/>
+      <c r="A7" s="61"/>
+      <c r="B7" s="60"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="23"/>
       <c r="G7" s="28"/>
       <c r="H7" s="29"/>
       <c r="I7" s="28"/>
@@ -20859,12 +21067,12 @@
       <c r="L7" s="33"/>
     </row>
     <row r="8" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="25"/>
-      <c r="B8" s="24"/>
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="41"/>
-      <c r="F8" s="42"/>
+      <c r="A8" s="61"/>
+      <c r="B8" s="60"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="25"/>
       <c r="G8" s="30"/>
       <c r="H8" s="31"/>
       <c r="I8" s="30"/>
@@ -20873,28 +21081,28 @@
       <c r="L8" s="34"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="48" t="s">
         <v>473</v>
       </c>
-      <c r="B9" s="13"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="38"/>
-      <c r="G9" s="43"/>
-      <c r="H9" s="44"/>
-      <c r="I9" s="43"/>
-      <c r="J9" s="44"/>
-      <c r="K9" s="43"/>
-      <c r="L9" s="45"/>
+      <c r="B9" s="49"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="27"/>
+      <c r="K9" s="26"/>
+      <c r="L9" s="32"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A10" s="14"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="36"/>
-      <c r="D10" s="36"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="40"/>
+      <c r="A10" s="50"/>
+      <c r="B10" s="49"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="23"/>
       <c r="G10" s="28"/>
       <c r="H10" s="29"/>
       <c r="I10" s="28"/>
@@ -20903,12 +21111,12 @@
       <c r="L10" s="33"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A11" s="14"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="36"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="41"/>
-      <c r="F11" s="42"/>
+      <c r="A11" s="50"/>
+      <c r="B11" s="49"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="25"/>
       <c r="G11" s="30"/>
       <c r="H11" s="31"/>
       <c r="I11" s="30"/>
@@ -20917,28 +21125,28 @@
       <c r="L11" s="34"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="48" t="s">
         <v>474</v>
       </c>
-      <c r="B12" s="13"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="37"/>
-      <c r="F12" s="38"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="44"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="44"/>
-      <c r="K12" s="43"/>
-      <c r="L12" s="45"/>
+      <c r="B12" s="49"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="26"/>
+      <c r="J12" s="27"/>
+      <c r="K12" s="26"/>
+      <c r="L12" s="32"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A13" s="14"/>
-      <c r="B13" s="13"/>
-      <c r="C13" s="36"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="40"/>
+      <c r="A13" s="50"/>
+      <c r="B13" s="49"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="23"/>
       <c r="G13" s="28"/>
       <c r="H13" s="29"/>
       <c r="I13" s="28"/>
@@ -20947,12 +21155,12 @@
       <c r="L13" s="33"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A14" s="14"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="41"/>
-      <c r="F14" s="42"/>
+      <c r="A14" s="50"/>
+      <c r="B14" s="49"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="25"/>
       <c r="G14" s="30"/>
       <c r="H14" s="31"/>
       <c r="I14" s="30"/>
@@ -20961,28 +21169,28 @@
       <c r="L14" s="34"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="48" t="s">
         <v>475</v>
       </c>
-      <c r="B15" s="13"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="38"/>
-      <c r="G15" s="43"/>
-      <c r="H15" s="44"/>
-      <c r="I15" s="43"/>
-      <c r="J15" s="44"/>
-      <c r="K15" s="43"/>
-      <c r="L15" s="45"/>
+      <c r="B15" s="49"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="26"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="26"/>
+      <c r="L15" s="32"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A16" s="14"/>
-      <c r="B16" s="13"/>
-      <c r="C16" s="36"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="40"/>
+      <c r="A16" s="50"/>
+      <c r="B16" s="49"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="23"/>
       <c r="G16" s="28"/>
       <c r="H16" s="29"/>
       <c r="I16" s="28"/>
@@ -20991,12 +21199,12 @@
       <c r="L16" s="33"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A17" s="14"/>
-      <c r="B17" s="13"/>
-      <c r="C17" s="36"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="41"/>
-      <c r="F17" s="42"/>
+      <c r="A17" s="50"/>
+      <c r="B17" s="49"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="25"/>
       <c r="G17" s="30"/>
       <c r="H17" s="31"/>
       <c r="I17" s="30"/>
@@ -21005,28 +21213,28 @@
       <c r="L17" s="34"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="48" t="s">
         <v>476</v>
       </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="38"/>
-      <c r="G18" s="43"/>
-      <c r="H18" s="44"/>
-      <c r="I18" s="43"/>
-      <c r="J18" s="44"/>
-      <c r="K18" s="43"/>
-      <c r="L18" s="45"/>
+      <c r="B18" s="49"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="26"/>
+      <c r="J18" s="27"/>
+      <c r="K18" s="26"/>
+      <c r="L18" s="32"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A19" s="14"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="36"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="40"/>
+      <c r="A19" s="50"/>
+      <c r="B19" s="49"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="23"/>
       <c r="G19" s="28"/>
       <c r="H19" s="29"/>
       <c r="I19" s="28"/>
@@ -21035,12 +21243,12 @@
       <c r="L19" s="33"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A20" s="14"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="36"/>
-      <c r="D20" s="36"/>
-      <c r="E20" s="41"/>
-      <c r="F20" s="42"/>
+      <c r="A20" s="50"/>
+      <c r="B20" s="49"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="25"/>
       <c r="G20" s="30"/>
       <c r="H20" s="31"/>
       <c r="I20" s="30"/>
@@ -21049,28 +21257,28 @@
       <c r="L20" s="34"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="48" t="s">
         <v>477</v>
       </c>
-      <c r="B21" s="13"/>
-      <c r="C21" s="35"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="38"/>
-      <c r="G21" s="43"/>
-      <c r="H21" s="44"/>
-      <c r="I21" s="43"/>
-      <c r="J21" s="44"/>
-      <c r="K21" s="43"/>
-      <c r="L21" s="45"/>
+      <c r="B21" s="49"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="26"/>
+      <c r="J21" s="27"/>
+      <c r="K21" s="26"/>
+      <c r="L21" s="32"/>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A22" s="14"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="36"/>
-      <c r="D22" s="36"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="40"/>
+      <c r="A22" s="50"/>
+      <c r="B22" s="49"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="23"/>
       <c r="G22" s="28"/>
       <c r="H22" s="29"/>
       <c r="I22" s="28"/>
@@ -21079,12 +21287,12 @@
       <c r="L22" s="33"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A23" s="14"/>
-      <c r="B23" s="13"/>
-      <c r="C23" s="36"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="41"/>
-      <c r="F23" s="42"/>
+      <c r="A23" s="50"/>
+      <c r="B23" s="49"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="25"/>
       <c r="G23" s="30"/>
       <c r="H23" s="31"/>
       <c r="I23" s="30"/>
@@ -21093,28 +21301,28 @@
       <c r="L23" s="34"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A24" s="12" t="s">
+      <c r="A24" s="48" t="s">
         <v>478</v>
       </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="37"/>
-      <c r="F24" s="38"/>
-      <c r="G24" s="43"/>
-      <c r="H24" s="44"/>
-      <c r="I24" s="43"/>
-      <c r="J24" s="44"/>
-      <c r="K24" s="43"/>
-      <c r="L24" s="45"/>
+      <c r="B24" s="49"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="26"/>
+      <c r="H24" s="27"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="27"/>
+      <c r="K24" s="26"/>
+      <c r="L24" s="32"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A25" s="14"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="36"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="39"/>
-      <c r="F25" s="40"/>
+      <c r="A25" s="50"/>
+      <c r="B25" s="49"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="23"/>
       <c r="G25" s="28"/>
       <c r="H25" s="29"/>
       <c r="I25" s="28"/>
@@ -21123,12 +21331,12 @@
       <c r="L25" s="33"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A26" s="14"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="36"/>
-      <c r="D26" s="36"/>
-      <c r="E26" s="41"/>
-      <c r="F26" s="42"/>
+      <c r="A26" s="50"/>
+      <c r="B26" s="49"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="25"/>
       <c r="G26" s="30"/>
       <c r="H26" s="31"/>
       <c r="I26" s="30"/>
@@ -21137,28 +21345,28 @@
       <c r="L26" s="34"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="48" t="s">
         <v>479</v>
       </c>
-      <c r="B27" s="13"/>
-      <c r="C27" s="35"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="37"/>
-      <c r="F27" s="38"/>
-      <c r="G27" s="43"/>
-      <c r="H27" s="44"/>
-      <c r="I27" s="43"/>
-      <c r="J27" s="44"/>
-      <c r="K27" s="43"/>
-      <c r="L27" s="45"/>
+      <c r="B27" s="49"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="26"/>
+      <c r="H27" s="27"/>
+      <c r="I27" s="26"/>
+      <c r="J27" s="27"/>
+      <c r="K27" s="26"/>
+      <c r="L27" s="32"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A28" s="14"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="36"/>
-      <c r="D28" s="36"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="40"/>
+      <c r="A28" s="50"/>
+      <c r="B28" s="49"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="23"/>
       <c r="G28" s="28"/>
       <c r="H28" s="29"/>
       <c r="I28" s="28"/>
@@ -21167,12 +21375,12 @@
       <c r="L28" s="33"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A29" s="14"/>
-      <c r="B29" s="13"/>
-      <c r="C29" s="36"/>
-      <c r="D29" s="36"/>
-      <c r="E29" s="41"/>
-      <c r="F29" s="42"/>
+      <c r="A29" s="50"/>
+      <c r="B29" s="49"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="25"/>
       <c r="G29" s="30"/>
       <c r="H29" s="31"/>
       <c r="I29" s="30"/>
@@ -21181,30 +21389,30 @@
       <c r="L29" s="34"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A30" s="12" t="s">
+      <c r="A30" s="48" t="s">
         <v>480</v>
       </c>
-      <c r="B30" s="13"/>
-      <c r="C30" s="35" t="s">
+      <c r="B30" s="49"/>
+      <c r="C30" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="D30" s="36"/>
-      <c r="E30" s="37"/>
-      <c r="F30" s="38"/>
-      <c r="G30" s="43"/>
-      <c r="H30" s="44"/>
-      <c r="I30" s="43"/>
-      <c r="J30" s="44"/>
-      <c r="K30" s="43"/>
-      <c r="L30" s="45"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="27"/>
+      <c r="I30" s="26"/>
+      <c r="J30" s="27"/>
+      <c r="K30" s="26"/>
+      <c r="L30" s="32"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A31" s="14"/>
-      <c r="B31" s="13"/>
-      <c r="C31" s="36"/>
-      <c r="D31" s="36"/>
-      <c r="E31" s="39"/>
-      <c r="F31" s="40"/>
+      <c r="A31" s="50"/>
+      <c r="B31" s="49"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="23"/>
       <c r="G31" s="28"/>
       <c r="H31" s="29"/>
       <c r="I31" s="28"/>
@@ -21213,77 +21421,21 @@
       <c r="L31" s="33"/>
     </row>
     <row r="32" spans="1:12" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="15"/>
-      <c r="B32" s="16"/>
-      <c r="C32" s="50"/>
-      <c r="D32" s="50"/>
-      <c r="E32" s="51"/>
-      <c r="F32" s="52"/>
-      <c r="G32" s="53"/>
-      <c r="H32" s="54"/>
-      <c r="I32" s="53"/>
-      <c r="J32" s="54"/>
-      <c r="K32" s="53"/>
-      <c r="L32" s="55"/>
+      <c r="A32" s="51"/>
+      <c r="B32" s="52"/>
+      <c r="C32" s="35"/>
+      <c r="D32" s="35"/>
+      <c r="E32" s="36"/>
+      <c r="F32" s="37"/>
+      <c r="G32" s="38"/>
+      <c r="H32" s="39"/>
+      <c r="I32" s="38"/>
+      <c r="J32" s="39"/>
+      <c r="K32" s="38"/>
+      <c r="L32" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="67">
-    <mergeCell ref="C1:L1"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="C27:D29"/>
-    <mergeCell ref="E27:F29"/>
-    <mergeCell ref="G27:H29"/>
-    <mergeCell ref="I27:J29"/>
-    <mergeCell ref="K27:L29"/>
-    <mergeCell ref="C30:D32"/>
-    <mergeCell ref="E30:F32"/>
-    <mergeCell ref="G30:H32"/>
-    <mergeCell ref="I30:J32"/>
-    <mergeCell ref="K30:L32"/>
-    <mergeCell ref="C21:D23"/>
-    <mergeCell ref="E21:F23"/>
-    <mergeCell ref="G21:H23"/>
-    <mergeCell ref="I21:J23"/>
-    <mergeCell ref="K21:L23"/>
-    <mergeCell ref="C24:D26"/>
-    <mergeCell ref="E24:F26"/>
-    <mergeCell ref="G24:H26"/>
-    <mergeCell ref="I24:J26"/>
-    <mergeCell ref="K24:L26"/>
-    <mergeCell ref="C15:D17"/>
-    <mergeCell ref="E15:F17"/>
-    <mergeCell ref="G15:H17"/>
-    <mergeCell ref="I15:J17"/>
-    <mergeCell ref="K15:L17"/>
-    <mergeCell ref="C18:D20"/>
-    <mergeCell ref="E18:F20"/>
-    <mergeCell ref="G18:H20"/>
-    <mergeCell ref="I18:J20"/>
-    <mergeCell ref="K18:L20"/>
-    <mergeCell ref="E9:F11"/>
-    <mergeCell ref="G9:H11"/>
-    <mergeCell ref="I9:J11"/>
-    <mergeCell ref="K9:L11"/>
-    <mergeCell ref="C12:D14"/>
-    <mergeCell ref="E12:F14"/>
-    <mergeCell ref="G12:H14"/>
-    <mergeCell ref="I12:J14"/>
-    <mergeCell ref="K12:L14"/>
-    <mergeCell ref="C9:D11"/>
-    <mergeCell ref="I3:J5"/>
-    <mergeCell ref="K3:L5"/>
-    <mergeCell ref="C6:D8"/>
-    <mergeCell ref="E6:F8"/>
-    <mergeCell ref="G6:H8"/>
-    <mergeCell ref="I6:J8"/>
-    <mergeCell ref="K6:L8"/>
-    <mergeCell ref="C3:D5"/>
-    <mergeCell ref="E3:F5"/>
-    <mergeCell ref="G3:H5"/>
     <mergeCell ref="A30:B32"/>
     <mergeCell ref="A1:B2"/>
     <mergeCell ref="A3:B5"/>
@@ -21295,6 +21447,62 @@
     <mergeCell ref="A21:B23"/>
     <mergeCell ref="A24:B26"/>
     <mergeCell ref="A27:B29"/>
+    <mergeCell ref="I3:J5"/>
+    <mergeCell ref="K3:L5"/>
+    <mergeCell ref="C6:D8"/>
+    <mergeCell ref="E6:F8"/>
+    <mergeCell ref="G6:H8"/>
+    <mergeCell ref="I6:J8"/>
+    <mergeCell ref="K6:L8"/>
+    <mergeCell ref="C3:D5"/>
+    <mergeCell ref="E3:F5"/>
+    <mergeCell ref="G3:H5"/>
+    <mergeCell ref="E9:F11"/>
+    <mergeCell ref="G9:H11"/>
+    <mergeCell ref="I9:J11"/>
+    <mergeCell ref="K9:L11"/>
+    <mergeCell ref="C12:D14"/>
+    <mergeCell ref="E12:F14"/>
+    <mergeCell ref="G12:H14"/>
+    <mergeCell ref="I12:J14"/>
+    <mergeCell ref="K12:L14"/>
+    <mergeCell ref="C9:D11"/>
+    <mergeCell ref="C18:D20"/>
+    <mergeCell ref="E18:F20"/>
+    <mergeCell ref="G18:H20"/>
+    <mergeCell ref="I18:J20"/>
+    <mergeCell ref="K18:L20"/>
+    <mergeCell ref="C15:D17"/>
+    <mergeCell ref="E15:F17"/>
+    <mergeCell ref="G15:H17"/>
+    <mergeCell ref="I15:J17"/>
+    <mergeCell ref="K15:L17"/>
+    <mergeCell ref="C24:D26"/>
+    <mergeCell ref="E24:F26"/>
+    <mergeCell ref="G24:H26"/>
+    <mergeCell ref="I24:J26"/>
+    <mergeCell ref="K24:L26"/>
+    <mergeCell ref="C21:D23"/>
+    <mergeCell ref="E21:F23"/>
+    <mergeCell ref="G21:H23"/>
+    <mergeCell ref="I21:J23"/>
+    <mergeCell ref="K21:L23"/>
+    <mergeCell ref="C30:D32"/>
+    <mergeCell ref="E30:F32"/>
+    <mergeCell ref="G30:H32"/>
+    <mergeCell ref="I30:J32"/>
+    <mergeCell ref="K30:L32"/>
+    <mergeCell ref="C27:D29"/>
+    <mergeCell ref="E27:F29"/>
+    <mergeCell ref="G27:H29"/>
+    <mergeCell ref="I27:J29"/>
+    <mergeCell ref="K27:L29"/>
+    <mergeCell ref="C1:L1"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="K2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Chapter 9 Quality completed
</commit_message>
<xml_diff>
--- a/PMBOK_ITTOs_Interactive_Dashboard_2025-09-12.xlsx
+++ b/PMBOK_ITTOs_Interactive_Dashboard_2025-09-12.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erichayes/Desktop/PMP/PMI/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erichayes/Documents/PMI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F642384B-4FE8-2349-8257-16900C6BC25D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86FF1554-8DA8-404C-87F3-598009E3FEA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="24220" windowHeight="16220" firstSheet="14" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" firstSheet="14" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Definitions" sheetId="16" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6186" uniqueCount="571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6208" uniqueCount="575">
   <si>
     <t>Process</t>
   </si>
@@ -2025,6 +2025,18 @@
 Role in project management: It allows you to track schedule variance, forecast completion dates, and manage stakeholder expectations</t>
     </r>
   </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
 </sst>
 </file>
 
@@ -2083,7 +2095,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2093,6 +2105,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2416,7 +2434,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2439,6 +2457,114 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2481,120 +2607,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -20547,133 +20566,177 @@
       <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="11"/>
+      <c r="B2" s="11" t="s">
+        <v>571</v>
+      </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>2</v>
       </c>
-      <c r="B3" s="11"/>
+      <c r="B3" s="11" t="s">
+        <v>572</v>
+      </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="11"/>
+      <c r="B4" s="11" t="s">
+        <v>572</v>
+      </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>4</v>
       </c>
-      <c r="B5" s="11"/>
+      <c r="B5" s="11" t="s">
+        <v>571</v>
+      </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>5</v>
       </c>
-      <c r="B6" s="11"/>
+      <c r="B6" s="11" t="s">
+        <v>572</v>
+      </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>6</v>
       </c>
-      <c r="B7" s="11"/>
+      <c r="B7" s="11" t="s">
+        <v>573</v>
+      </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>7</v>
       </c>
-      <c r="B8" s="11"/>
+      <c r="B8" s="11" t="s">
+        <v>572</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>8</v>
       </c>
-      <c r="B9" s="11"/>
+      <c r="B9" s="64" t="s">
+        <v>572</v>
+      </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>9</v>
       </c>
-      <c r="B10" s="11"/>
+      <c r="B10" s="11" t="s">
+        <v>572</v>
+      </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>10</v>
       </c>
-      <c r="B11" s="11"/>
+      <c r="B11" s="11" t="s">
+        <v>571</v>
+      </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>11</v>
       </c>
-      <c r="B12" s="11"/>
+      <c r="B12" s="11" t="s">
+        <v>572</v>
+      </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>12</v>
       </c>
-      <c r="B13" s="11"/>
+      <c r="B13" s="11" t="s">
+        <v>572</v>
+      </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>13</v>
       </c>
-      <c r="B14" s="11"/>
+      <c r="B14" s="64" t="s">
+        <v>572</v>
+      </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>14</v>
       </c>
-      <c r="B15" s="11"/>
+      <c r="B15" s="64" t="s">
+        <v>574</v>
+      </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>15</v>
       </c>
-      <c r="B16" s="11"/>
+      <c r="B16" s="11" t="s">
+        <v>571</v>
+      </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>16</v>
       </c>
-      <c r="B17" s="11"/>
+      <c r="B17" s="11" t="s">
+        <v>574</v>
+      </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>17</v>
       </c>
-      <c r="B18" s="11"/>
+      <c r="B18" s="11" t="s">
+        <v>573</v>
+      </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>18</v>
       </c>
-      <c r="B19" s="11"/>
+      <c r="B19" s="11" t="s">
+        <v>574</v>
+      </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>19</v>
       </c>
-      <c r="B20" s="11"/>
+      <c r="B20" s="11" t="s">
+        <v>573</v>
+      </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>20</v>
       </c>
-      <c r="B21" s="11"/>
+      <c r="B21" s="11" t="s">
+        <v>571</v>
+      </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>21</v>
       </c>
-      <c r="B22" s="11"/>
+      <c r="B22" s="11" t="s">
+        <v>571</v>
+      </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>22</v>
       </c>
-      <c r="B23" s="11"/>
+      <c r="B23" s="11" t="s">
+        <v>571</v>
+      </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
@@ -20728,8 +20791,8 @@
         <v>568</v>
       </c>
       <c r="C33" s="8">
-        <f>1-(9/27)</f>
-        <v>0.66666666666666674</v>
+        <f>1-(3/22)</f>
+        <v>0.86363636363636365</v>
       </c>
     </row>
   </sheetData>
@@ -20750,74 +20813,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="22" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="53" t="s">
         <v>469</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="56" t="s">
+      <c r="B1" s="54"/>
+      <c r="C1" s="12" t="s">
         <v>470</v>
       </c>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
-      <c r="L1" s="58"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="14"/>
     </row>
     <row r="2" spans="1:12" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="19"/>
-      <c r="B2" s="20"/>
-      <c r="C2" s="59" t="s">
+      <c r="A2" s="55"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="60"/>
-      <c r="E2" s="59" t="s">
-        <v>57</v>
-      </c>
-      <c r="F2" s="60"/>
-      <c r="G2" s="59" t="s">
+      <c r="D2" s="16"/>
+      <c r="E2" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="16"/>
+      <c r="G2" s="15" t="s">
         <v>249</v>
       </c>
-      <c r="H2" s="60"/>
-      <c r="I2" s="61" t="s">
+      <c r="H2" s="16"/>
+      <c r="I2" s="17" t="s">
         <v>481</v>
       </c>
-      <c r="J2" s="60"/>
-      <c r="K2" s="59" t="s">
+      <c r="J2" s="16"/>
+      <c r="K2" s="15" t="s">
         <v>377</v>
       </c>
-      <c r="L2" s="60"/>
+      <c r="L2" s="16"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="57" t="s">
         <v>471</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="46" t="s">
+      <c r="B3" s="58"/>
+      <c r="C3" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="47"/>
-      <c r="E3" s="48" t="s">
+      <c r="D3" s="45"/>
+      <c r="E3" s="46" t="s">
         <v>56</v>
       </c>
-      <c r="F3" s="49"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="27"/>
-      <c r="I3" s="26"/>
-      <c r="J3" s="27"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="32"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="42"/>
+      <c r="I3" s="41"/>
+      <c r="J3" s="42"/>
+      <c r="K3" s="41"/>
+      <c r="L3" s="43"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A4" s="14"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="40"/>
+      <c r="A4" s="50"/>
+      <c r="B4" s="49"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="23"/>
       <c r="G4" s="28"/>
       <c r="H4" s="29"/>
       <c r="I4" s="28"/>
@@ -20826,12 +20889,12 @@
       <c r="L4" s="33"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" s="14"/>
-      <c r="B5" s="13"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="41"/>
-      <c r="F5" s="42"/>
+      <c r="A5" s="50"/>
+      <c r="B5" s="49"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="25"/>
       <c r="G5" s="30"/>
       <c r="H5" s="31"/>
       <c r="I5" s="30"/>
@@ -20840,30 +20903,30 @@
       <c r="L5" s="34"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="59" t="s">
         <v>472</v>
       </c>
-      <c r="B6" s="24"/>
-      <c r="C6" s="35"/>
-      <c r="D6" s="36"/>
-      <c r="E6" s="37" t="s">
+      <c r="B6" s="60"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="20" t="s">
         <v>482</v>
       </c>
-      <c r="F6" s="38"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
-      <c r="I6" s="43"/>
-      <c r="J6" s="44"/>
-      <c r="K6" s="43"/>
-      <c r="L6" s="45"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="27"/>
+      <c r="K6" s="26"/>
+      <c r="L6" s="32"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="25"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="40"/>
+      <c r="A7" s="61"/>
+      <c r="B7" s="60"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="23"/>
       <c r="G7" s="28"/>
       <c r="H7" s="29"/>
       <c r="I7" s="28"/>
@@ -20872,12 +20935,12 @@
       <c r="L7" s="33"/>
     </row>
     <row r="8" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="25"/>
-      <c r="B8" s="24"/>
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="41"/>
-      <c r="F8" s="42"/>
+      <c r="A8" s="61"/>
+      <c r="B8" s="60"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="25"/>
       <c r="G8" s="30"/>
       <c r="H8" s="31"/>
       <c r="I8" s="30"/>
@@ -20886,28 +20949,28 @@
       <c r="L8" s="34"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="48" t="s">
         <v>473</v>
       </c>
-      <c r="B9" s="13"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="38"/>
-      <c r="G9" s="43"/>
-      <c r="H9" s="44"/>
-      <c r="I9" s="43"/>
-      <c r="J9" s="44"/>
-      <c r="K9" s="43"/>
-      <c r="L9" s="45"/>
+      <c r="B9" s="49"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="27"/>
+      <c r="K9" s="26"/>
+      <c r="L9" s="32"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" s="14"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="36"/>
-      <c r="D10" s="36"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="40"/>
+      <c r="A10" s="50"/>
+      <c r="B10" s="49"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="23"/>
       <c r="G10" s="28"/>
       <c r="H10" s="29"/>
       <c r="I10" s="28"/>
@@ -20916,12 +20979,12 @@
       <c r="L10" s="33"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A11" s="14"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="36"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="41"/>
-      <c r="F11" s="42"/>
+      <c r="A11" s="50"/>
+      <c r="B11" s="49"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="25"/>
       <c r="G11" s="30"/>
       <c r="H11" s="31"/>
       <c r="I11" s="30"/>
@@ -20930,28 +20993,28 @@
       <c r="L11" s="34"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="48" t="s">
         <v>474</v>
       </c>
-      <c r="B12" s="13"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="37"/>
-      <c r="F12" s="38"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="44"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="44"/>
-      <c r="K12" s="43"/>
-      <c r="L12" s="45"/>
+      <c r="B12" s="49"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="26"/>
+      <c r="J12" s="27"/>
+      <c r="K12" s="26"/>
+      <c r="L12" s="32"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A13" s="14"/>
-      <c r="B13" s="13"/>
-      <c r="C13" s="36"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="40"/>
+      <c r="A13" s="50"/>
+      <c r="B13" s="49"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="23"/>
       <c r="G13" s="28"/>
       <c r="H13" s="29"/>
       <c r="I13" s="28"/>
@@ -20960,12 +21023,12 @@
       <c r="L13" s="33"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A14" s="14"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="41"/>
-      <c r="F14" s="42"/>
+      <c r="A14" s="50"/>
+      <c r="B14" s="49"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="25"/>
       <c r="G14" s="30"/>
       <c r="H14" s="31"/>
       <c r="I14" s="30"/>
@@ -20974,28 +21037,28 @@
       <c r="L14" s="34"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="48" t="s">
         <v>475</v>
       </c>
-      <c r="B15" s="13"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="38"/>
-      <c r="G15" s="43"/>
-      <c r="H15" s="44"/>
-      <c r="I15" s="43"/>
-      <c r="J15" s="44"/>
-      <c r="K15" s="43"/>
-      <c r="L15" s="45"/>
+      <c r="B15" s="49"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="26"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="26"/>
+      <c r="L15" s="32"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A16" s="14"/>
-      <c r="B16" s="13"/>
-      <c r="C16" s="36"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="40"/>
+      <c r="A16" s="50"/>
+      <c r="B16" s="49"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="23"/>
       <c r="G16" s="28"/>
       <c r="H16" s="29"/>
       <c r="I16" s="28"/>
@@ -21004,12 +21067,12 @@
       <c r="L16" s="33"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A17" s="14"/>
-      <c r="B17" s="13"/>
-      <c r="C17" s="36"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="41"/>
-      <c r="F17" s="42"/>
+      <c r="A17" s="50"/>
+      <c r="B17" s="49"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="25"/>
       <c r="G17" s="30"/>
       <c r="H17" s="31"/>
       <c r="I17" s="30"/>
@@ -21018,28 +21081,28 @@
       <c r="L17" s="34"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="48" t="s">
         <v>476</v>
       </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="38"/>
-      <c r="G18" s="43"/>
-      <c r="H18" s="44"/>
-      <c r="I18" s="43"/>
-      <c r="J18" s="44"/>
-      <c r="K18" s="43"/>
-      <c r="L18" s="45"/>
+      <c r="B18" s="49"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="26"/>
+      <c r="J18" s="27"/>
+      <c r="K18" s="26"/>
+      <c r="L18" s="32"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A19" s="14"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="36"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="40"/>
+      <c r="A19" s="50"/>
+      <c r="B19" s="49"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="23"/>
       <c r="G19" s="28"/>
       <c r="H19" s="29"/>
       <c r="I19" s="28"/>
@@ -21048,12 +21111,12 @@
       <c r="L19" s="33"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A20" s="14"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="36"/>
-      <c r="D20" s="36"/>
-      <c r="E20" s="41"/>
-      <c r="F20" s="42"/>
+      <c r="A20" s="50"/>
+      <c r="B20" s="49"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="25"/>
       <c r="G20" s="30"/>
       <c r="H20" s="31"/>
       <c r="I20" s="30"/>
@@ -21062,28 +21125,28 @@
       <c r="L20" s="34"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="48" t="s">
         <v>477</v>
       </c>
-      <c r="B21" s="13"/>
-      <c r="C21" s="35"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="38"/>
-      <c r="G21" s="43"/>
-      <c r="H21" s="44"/>
-      <c r="I21" s="43"/>
-      <c r="J21" s="44"/>
-      <c r="K21" s="43"/>
-      <c r="L21" s="45"/>
+      <c r="B21" s="49"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="26"/>
+      <c r="J21" s="27"/>
+      <c r="K21" s="26"/>
+      <c r="L21" s="32"/>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A22" s="14"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="36"/>
-      <c r="D22" s="36"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="40"/>
+      <c r="A22" s="50"/>
+      <c r="B22" s="49"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="23"/>
       <c r="G22" s="28"/>
       <c r="H22" s="29"/>
       <c r="I22" s="28"/>
@@ -21092,12 +21155,12 @@
       <c r="L22" s="33"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A23" s="14"/>
-      <c r="B23" s="13"/>
-      <c r="C23" s="36"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="41"/>
-      <c r="F23" s="42"/>
+      <c r="A23" s="50"/>
+      <c r="B23" s="49"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="25"/>
       <c r="G23" s="30"/>
       <c r="H23" s="31"/>
       <c r="I23" s="30"/>
@@ -21106,28 +21169,28 @@
       <c r="L23" s="34"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A24" s="12" t="s">
+      <c r="A24" s="48" t="s">
         <v>478</v>
       </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="37"/>
-      <c r="F24" s="38"/>
-      <c r="G24" s="43"/>
-      <c r="H24" s="44"/>
-      <c r="I24" s="43"/>
-      <c r="J24" s="44"/>
-      <c r="K24" s="43"/>
-      <c r="L24" s="45"/>
+      <c r="B24" s="49"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="26"/>
+      <c r="H24" s="27"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="27"/>
+      <c r="K24" s="26"/>
+      <c r="L24" s="32"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A25" s="14"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="36"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="39"/>
-      <c r="F25" s="40"/>
+      <c r="A25" s="50"/>
+      <c r="B25" s="49"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="23"/>
       <c r="G25" s="28"/>
       <c r="H25" s="29"/>
       <c r="I25" s="28"/>
@@ -21136,12 +21199,12 @@
       <c r="L25" s="33"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A26" s="14"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="36"/>
-      <c r="D26" s="36"/>
-      <c r="E26" s="41"/>
-      <c r="F26" s="42"/>
+      <c r="A26" s="50"/>
+      <c r="B26" s="49"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="25"/>
       <c r="G26" s="30"/>
       <c r="H26" s="31"/>
       <c r="I26" s="30"/>
@@ -21150,28 +21213,28 @@
       <c r="L26" s="34"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="48" t="s">
         <v>479</v>
       </c>
-      <c r="B27" s="13"/>
-      <c r="C27" s="35"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="37"/>
-      <c r="F27" s="38"/>
-      <c r="G27" s="43"/>
-      <c r="H27" s="44"/>
-      <c r="I27" s="43"/>
-      <c r="J27" s="44"/>
-      <c r="K27" s="43"/>
-      <c r="L27" s="45"/>
+      <c r="B27" s="49"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="26"/>
+      <c r="H27" s="27"/>
+      <c r="I27" s="26"/>
+      <c r="J27" s="27"/>
+      <c r="K27" s="26"/>
+      <c r="L27" s="32"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A28" s="14"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="36"/>
-      <c r="D28" s="36"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="40"/>
+      <c r="A28" s="50"/>
+      <c r="B28" s="49"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="23"/>
       <c r="G28" s="28"/>
       <c r="H28" s="29"/>
       <c r="I28" s="28"/>
@@ -21180,12 +21243,12 @@
       <c r="L28" s="33"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A29" s="14"/>
-      <c r="B29" s="13"/>
-      <c r="C29" s="36"/>
-      <c r="D29" s="36"/>
-      <c r="E29" s="41"/>
-      <c r="F29" s="42"/>
+      <c r="A29" s="50"/>
+      <c r="B29" s="49"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="25"/>
       <c r="G29" s="30"/>
       <c r="H29" s="31"/>
       <c r="I29" s="30"/>
@@ -21194,30 +21257,30 @@
       <c r="L29" s="34"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A30" s="12" t="s">
+      <c r="A30" s="48" t="s">
         <v>480</v>
       </c>
-      <c r="B30" s="13"/>
-      <c r="C30" s="35" t="s">
+      <c r="B30" s="49"/>
+      <c r="C30" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="D30" s="36"/>
-      <c r="E30" s="37"/>
-      <c r="F30" s="38"/>
-      <c r="G30" s="43"/>
-      <c r="H30" s="44"/>
-      <c r="I30" s="43"/>
-      <c r="J30" s="44"/>
-      <c r="K30" s="43"/>
-      <c r="L30" s="45"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="27"/>
+      <c r="I30" s="26"/>
+      <c r="J30" s="27"/>
+      <c r="K30" s="26"/>
+      <c r="L30" s="32"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A31" s="14"/>
-      <c r="B31" s="13"/>
-      <c r="C31" s="36"/>
-      <c r="D31" s="36"/>
-      <c r="E31" s="39"/>
-      <c r="F31" s="40"/>
+      <c r="A31" s="50"/>
+      <c r="B31" s="49"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="23"/>
       <c r="G31" s="28"/>
       <c r="H31" s="29"/>
       <c r="I31" s="28"/>
@@ -21226,77 +21289,21 @@
       <c r="L31" s="33"/>
     </row>
     <row r="32" spans="1:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="15"/>
-      <c r="B32" s="16"/>
-      <c r="C32" s="50"/>
-      <c r="D32" s="50"/>
-      <c r="E32" s="51"/>
-      <c r="F32" s="52"/>
-      <c r="G32" s="53"/>
-      <c r="H32" s="54"/>
-      <c r="I32" s="53"/>
-      <c r="J32" s="54"/>
-      <c r="K32" s="53"/>
-      <c r="L32" s="55"/>
+      <c r="A32" s="51"/>
+      <c r="B32" s="52"/>
+      <c r="C32" s="35"/>
+      <c r="D32" s="35"/>
+      <c r="E32" s="36"/>
+      <c r="F32" s="37"/>
+      <c r="G32" s="38"/>
+      <c r="H32" s="39"/>
+      <c r="I32" s="38"/>
+      <c r="J32" s="39"/>
+      <c r="K32" s="38"/>
+      <c r="L32" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="67">
-    <mergeCell ref="C1:L1"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="C27:D29"/>
-    <mergeCell ref="E27:F29"/>
-    <mergeCell ref="G27:H29"/>
-    <mergeCell ref="I27:J29"/>
-    <mergeCell ref="K27:L29"/>
-    <mergeCell ref="C30:D32"/>
-    <mergeCell ref="E30:F32"/>
-    <mergeCell ref="G30:H32"/>
-    <mergeCell ref="I30:J32"/>
-    <mergeCell ref="K30:L32"/>
-    <mergeCell ref="C21:D23"/>
-    <mergeCell ref="E21:F23"/>
-    <mergeCell ref="G21:H23"/>
-    <mergeCell ref="I21:J23"/>
-    <mergeCell ref="K21:L23"/>
-    <mergeCell ref="C24:D26"/>
-    <mergeCell ref="E24:F26"/>
-    <mergeCell ref="G24:H26"/>
-    <mergeCell ref="I24:J26"/>
-    <mergeCell ref="K24:L26"/>
-    <mergeCell ref="C15:D17"/>
-    <mergeCell ref="E15:F17"/>
-    <mergeCell ref="G15:H17"/>
-    <mergeCell ref="I15:J17"/>
-    <mergeCell ref="K15:L17"/>
-    <mergeCell ref="C18:D20"/>
-    <mergeCell ref="E18:F20"/>
-    <mergeCell ref="G18:H20"/>
-    <mergeCell ref="I18:J20"/>
-    <mergeCell ref="K18:L20"/>
-    <mergeCell ref="E9:F11"/>
-    <mergeCell ref="G9:H11"/>
-    <mergeCell ref="I9:J11"/>
-    <mergeCell ref="K9:L11"/>
-    <mergeCell ref="C12:D14"/>
-    <mergeCell ref="E12:F14"/>
-    <mergeCell ref="G12:H14"/>
-    <mergeCell ref="I12:J14"/>
-    <mergeCell ref="K12:L14"/>
-    <mergeCell ref="C9:D11"/>
-    <mergeCell ref="I3:J5"/>
-    <mergeCell ref="K3:L5"/>
-    <mergeCell ref="C6:D8"/>
-    <mergeCell ref="E6:F8"/>
-    <mergeCell ref="G6:H8"/>
-    <mergeCell ref="I6:J8"/>
-    <mergeCell ref="K6:L8"/>
-    <mergeCell ref="C3:D5"/>
-    <mergeCell ref="E3:F5"/>
-    <mergeCell ref="G3:H5"/>
     <mergeCell ref="A30:B32"/>
     <mergeCell ref="A1:B2"/>
     <mergeCell ref="A3:B5"/>
@@ -21308,6 +21315,62 @@
     <mergeCell ref="A21:B23"/>
     <mergeCell ref="A24:B26"/>
     <mergeCell ref="A27:B29"/>
+    <mergeCell ref="I3:J5"/>
+    <mergeCell ref="K3:L5"/>
+    <mergeCell ref="C6:D8"/>
+    <mergeCell ref="E6:F8"/>
+    <mergeCell ref="G6:H8"/>
+    <mergeCell ref="I6:J8"/>
+    <mergeCell ref="K6:L8"/>
+    <mergeCell ref="C3:D5"/>
+    <mergeCell ref="E3:F5"/>
+    <mergeCell ref="G3:H5"/>
+    <mergeCell ref="E9:F11"/>
+    <mergeCell ref="G9:H11"/>
+    <mergeCell ref="I9:J11"/>
+    <mergeCell ref="K9:L11"/>
+    <mergeCell ref="C12:D14"/>
+    <mergeCell ref="E12:F14"/>
+    <mergeCell ref="G12:H14"/>
+    <mergeCell ref="I12:J14"/>
+    <mergeCell ref="K12:L14"/>
+    <mergeCell ref="C9:D11"/>
+    <mergeCell ref="C18:D20"/>
+    <mergeCell ref="E18:F20"/>
+    <mergeCell ref="G18:H20"/>
+    <mergeCell ref="I18:J20"/>
+    <mergeCell ref="K18:L20"/>
+    <mergeCell ref="C15:D17"/>
+    <mergeCell ref="E15:F17"/>
+    <mergeCell ref="G15:H17"/>
+    <mergeCell ref="I15:J17"/>
+    <mergeCell ref="K15:L17"/>
+    <mergeCell ref="C24:D26"/>
+    <mergeCell ref="E24:F26"/>
+    <mergeCell ref="G24:H26"/>
+    <mergeCell ref="I24:J26"/>
+    <mergeCell ref="K24:L26"/>
+    <mergeCell ref="C21:D23"/>
+    <mergeCell ref="E21:F23"/>
+    <mergeCell ref="G21:H23"/>
+    <mergeCell ref="I21:J23"/>
+    <mergeCell ref="K21:L23"/>
+    <mergeCell ref="C30:D32"/>
+    <mergeCell ref="E30:F32"/>
+    <mergeCell ref="G30:H32"/>
+    <mergeCell ref="I30:J32"/>
+    <mergeCell ref="K30:L32"/>
+    <mergeCell ref="C27:D29"/>
+    <mergeCell ref="E27:F29"/>
+    <mergeCell ref="G27:H29"/>
+    <mergeCell ref="I27:J29"/>
+    <mergeCell ref="K27:L29"/>
+    <mergeCell ref="C1:L1"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="K2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Chapter 13 Procurement Managment
</commit_message>
<xml_diff>
--- a/PMBOK_ITTOs_Interactive_Dashboard_2025-09-12.xlsx
+++ b/PMBOK_ITTOs_Interactive_Dashboard_2025-09-12.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eric.hayes\Documents\PMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78254B08-DF30-4E14-A49A-C4BF7E0BC8B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6049211C-FB81-4B99-A1C0-E214261E6175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11910" yWindow="0" windowWidth="12180" windowHeight="16090" firstSheet="18" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="16220" firstSheet="20" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Definitions" sheetId="16" r:id="rId1"/>
@@ -34,7 +34,9 @@
     <sheet name="CH10 Project Resource Managemen" sheetId="20" r:id="rId19"/>
     <sheet name="CH11 Project Comms Manag" sheetId="22" r:id="rId20"/>
     <sheet name="CH12 Project Risk Managment" sheetId="23" r:id="rId21"/>
-    <sheet name="Sheet3" sheetId="21" r:id="rId22"/>
+    <sheet name="CH13 Project Procure Managment" sheetId="24" r:id="rId22"/>
+    <sheet name="CH14 Project STKHLDR Managm" sheetId="25" r:id="rId23"/>
+    <sheet name="Sheet3" sheetId="21" r:id="rId24"/>
   </sheets>
   <definedNames>
     <definedName name="Slicer_ITTO_Name">#N/A</definedName>
@@ -48,9 +50,9 @@
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{46BE6895-7355-4a93-B00E-2C351335B9C9}">
       <x15:slicerCaches xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
-        <x14:slicerCache r:id="rId23"/>
-        <x14:slicerCache r:id="rId24"/>
         <x14:slicerCache r:id="rId25"/>
+        <x14:slicerCache r:id="rId26"/>
+        <x14:slicerCache r:id="rId27"/>
       </x15:slicerCaches>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -69,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6323" uniqueCount="577">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6358" uniqueCount="577">
   <si>
     <t>Process</t>
   </si>
@@ -2483,6 +2485,114 @@
       </extLst>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2524,114 +2634,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -21195,74 +21197,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="56" t="s">
         <v>469</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="59" t="s">
+      <c r="B1" s="57"/>
+      <c r="C1" s="15" t="s">
         <v>470</v>
       </c>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="61"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="17"/>
     </row>
     <row r="2" spans="1:12" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="22"/>
-      <c r="B2" s="23"/>
-      <c r="C2" s="62" t="s">
+      <c r="A2" s="58"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="63"/>
-      <c r="E2" s="62" t="s">
-        <v>57</v>
-      </c>
-      <c r="F2" s="63"/>
-      <c r="G2" s="62" t="s">
+      <c r="D2" s="19"/>
+      <c r="E2" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="19"/>
+      <c r="G2" s="18" t="s">
         <v>249</v>
       </c>
-      <c r="H2" s="63"/>
-      <c r="I2" s="64" t="s">
+      <c r="H2" s="19"/>
+      <c r="I2" s="20" t="s">
         <v>481</v>
       </c>
-      <c r="J2" s="63"/>
-      <c r="K2" s="62" t="s">
+      <c r="J2" s="19"/>
+      <c r="K2" s="18" t="s">
         <v>377</v>
       </c>
-      <c r="L2" s="63"/>
+      <c r="L2" s="19"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="60" t="s">
         <v>471</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="49" t="s">
+      <c r="B3" s="61"/>
+      <c r="C3" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="50"/>
-      <c r="E3" s="51" t="s">
+      <c r="D3" s="48"/>
+      <c r="E3" s="49" t="s">
         <v>56</v>
       </c>
-      <c r="F3" s="52"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="35"/>
+      <c r="F3" s="50"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="45"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="45"/>
+      <c r="K3" s="44"/>
+      <c r="L3" s="46"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A4" s="17"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="43"/>
+      <c r="A4" s="53"/>
+      <c r="B4" s="52"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="26"/>
       <c r="G4" s="31"/>
       <c r="H4" s="32"/>
       <c r="I4" s="31"/>
@@ -21271,12 +21273,12 @@
       <c r="L4" s="36"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A5" s="17"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="45"/>
+      <c r="A5" s="53"/>
+      <c r="B5" s="52"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="28"/>
       <c r="G5" s="33"/>
       <c r="H5" s="34"/>
       <c r="I5" s="33"/>
@@ -21285,30 +21287,30 @@
       <c r="L5" s="37"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A6" s="26" t="s">
+      <c r="A6" s="62" t="s">
         <v>472</v>
       </c>
-      <c r="B6" s="27"/>
-      <c r="C6" s="38"/>
-      <c r="D6" s="39"/>
-      <c r="E6" s="40" t="s">
+      <c r="B6" s="63"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="23" t="s">
         <v>482</v>
       </c>
-      <c r="F6" s="41"/>
-      <c r="G6" s="46"/>
-      <c r="H6" s="47"/>
-      <c r="I6" s="46"/>
-      <c r="J6" s="47"/>
-      <c r="K6" s="46"/>
-      <c r="L6" s="48"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="29"/>
+      <c r="J6" s="30"/>
+      <c r="K6" s="29"/>
+      <c r="L6" s="35"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A7" s="28"/>
-      <c r="B7" s="27"/>
-      <c r="C7" s="39"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="42"/>
-      <c r="F7" s="43"/>
+      <c r="A7" s="64"/>
+      <c r="B7" s="63"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="26"/>
       <c r="G7" s="31"/>
       <c r="H7" s="32"/>
       <c r="I7" s="31"/>
@@ -21317,12 +21319,12 @@
       <c r="L7" s="36"/>
     </row>
     <row r="8" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="28"/>
-      <c r="B8" s="27"/>
-      <c r="C8" s="39"/>
-      <c r="D8" s="39"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="45"/>
+      <c r="A8" s="64"/>
+      <c r="B8" s="63"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="28"/>
       <c r="G8" s="33"/>
       <c r="H8" s="34"/>
       <c r="I8" s="33"/>
@@ -21331,28 +21333,28 @@
       <c r="L8" s="37"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="51" t="s">
         <v>473</v>
       </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="38"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="40"/>
-      <c r="F9" s="41"/>
-      <c r="G9" s="46"/>
-      <c r="H9" s="47"/>
-      <c r="I9" s="46"/>
-      <c r="J9" s="47"/>
-      <c r="K9" s="46"/>
-      <c r="L9" s="48"/>
+      <c r="B9" s="52"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="29"/>
+      <c r="J9" s="30"/>
+      <c r="K9" s="29"/>
+      <c r="L9" s="35"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A10" s="17"/>
-      <c r="B10" s="16"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="42"/>
-      <c r="F10" s="43"/>
+      <c r="A10" s="53"/>
+      <c r="B10" s="52"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="26"/>
       <c r="G10" s="31"/>
       <c r="H10" s="32"/>
       <c r="I10" s="31"/>
@@ -21361,12 +21363,12 @@
       <c r="L10" s="36"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A11" s="17"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="44"/>
-      <c r="F11" s="45"/>
+      <c r="A11" s="53"/>
+      <c r="B11" s="52"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="28"/>
       <c r="G11" s="33"/>
       <c r="H11" s="34"/>
       <c r="I11" s="33"/>
@@ -21375,28 +21377,28 @@
       <c r="L11" s="37"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="51" t="s">
         <v>474</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="40"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="46"/>
-      <c r="H12" s="47"/>
-      <c r="I12" s="46"/>
-      <c r="J12" s="47"/>
-      <c r="K12" s="46"/>
-      <c r="L12" s="48"/>
+      <c r="B12" s="52"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="29"/>
+      <c r="J12" s="30"/>
+      <c r="K12" s="29"/>
+      <c r="L12" s="35"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A13" s="17"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="39"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="42"/>
-      <c r="F13" s="43"/>
+      <c r="A13" s="53"/>
+      <c r="B13" s="52"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="26"/>
       <c r="G13" s="31"/>
       <c r="H13" s="32"/>
       <c r="I13" s="31"/>
@@ -21405,12 +21407,12 @@
       <c r="L13" s="36"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A14" s="17"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="39"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="45"/>
+      <c r="A14" s="53"/>
+      <c r="B14" s="52"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="28"/>
       <c r="G14" s="33"/>
       <c r="H14" s="34"/>
       <c r="I14" s="33"/>
@@ -21419,28 +21421,28 @@
       <c r="L14" s="37"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="51" t="s">
         <v>475</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="41"/>
-      <c r="G15" s="46"/>
-      <c r="H15" s="47"/>
-      <c r="I15" s="46"/>
-      <c r="J15" s="47"/>
-      <c r="K15" s="46"/>
-      <c r="L15" s="48"/>
+      <c r="B15" s="52"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="29"/>
+      <c r="J15" s="30"/>
+      <c r="K15" s="29"/>
+      <c r="L15" s="35"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A16" s="17"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="39"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="42"/>
-      <c r="F16" s="43"/>
+      <c r="A16" s="53"/>
+      <c r="B16" s="52"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="26"/>
       <c r="G16" s="31"/>
       <c r="H16" s="32"/>
       <c r="I16" s="31"/>
@@ -21449,12 +21451,12 @@
       <c r="L16" s="36"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A17" s="17"/>
-      <c r="B17" s="16"/>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="44"/>
-      <c r="F17" s="45"/>
+      <c r="A17" s="53"/>
+      <c r="B17" s="52"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="28"/>
       <c r="G17" s="33"/>
       <c r="H17" s="34"/>
       <c r="I17" s="33"/>
@@ -21463,28 +21465,28 @@
       <c r="L17" s="37"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A18" s="15" t="s">
+      <c r="A18" s="51" t="s">
         <v>476</v>
       </c>
-      <c r="B18" s="16"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="40"/>
-      <c r="F18" s="41"/>
-      <c r="G18" s="46"/>
-      <c r="H18" s="47"/>
-      <c r="I18" s="46"/>
-      <c r="J18" s="47"/>
-      <c r="K18" s="46"/>
-      <c r="L18" s="48"/>
+      <c r="B18" s="52"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="29"/>
+      <c r="J18" s="30"/>
+      <c r="K18" s="29"/>
+      <c r="L18" s="35"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A19" s="17"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="39"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="42"/>
-      <c r="F19" s="43"/>
+      <c r="A19" s="53"/>
+      <c r="B19" s="52"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="25"/>
+      <c r="F19" s="26"/>
       <c r="G19" s="31"/>
       <c r="H19" s="32"/>
       <c r="I19" s="31"/>
@@ -21493,12 +21495,12 @@
       <c r="L19" s="36"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A20" s="17"/>
-      <c r="B20" s="16"/>
-      <c r="C20" s="39"/>
-      <c r="D20" s="39"/>
-      <c r="E20" s="44"/>
-      <c r="F20" s="45"/>
+      <c r="A20" s="53"/>
+      <c r="B20" s="52"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="28"/>
       <c r="G20" s="33"/>
       <c r="H20" s="34"/>
       <c r="I20" s="33"/>
@@ -21507,28 +21509,28 @@
       <c r="L20" s="37"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A21" s="15" t="s">
+      <c r="A21" s="51" t="s">
         <v>477</v>
       </c>
-      <c r="B21" s="16"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="39"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="46"/>
-      <c r="H21" s="47"/>
-      <c r="I21" s="46"/>
-      <c r="J21" s="47"/>
-      <c r="K21" s="46"/>
-      <c r="L21" s="48"/>
+      <c r="B21" s="52"/>
+      <c r="C21" s="21"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="30"/>
+      <c r="I21" s="29"/>
+      <c r="J21" s="30"/>
+      <c r="K21" s="29"/>
+      <c r="L21" s="35"/>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A22" s="17"/>
-      <c r="B22" s="16"/>
-      <c r="C22" s="39"/>
-      <c r="D22" s="39"/>
-      <c r="E22" s="42"/>
-      <c r="F22" s="43"/>
+      <c r="A22" s="53"/>
+      <c r="B22" s="52"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="26"/>
       <c r="G22" s="31"/>
       <c r="H22" s="32"/>
       <c r="I22" s="31"/>
@@ -21537,12 +21539,12 @@
       <c r="L22" s="36"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A23" s="17"/>
-      <c r="B23" s="16"/>
-      <c r="C23" s="39"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="44"/>
-      <c r="F23" s="45"/>
+      <c r="A23" s="53"/>
+      <c r="B23" s="52"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="28"/>
       <c r="G23" s="33"/>
       <c r="H23" s="34"/>
       <c r="I23" s="33"/>
@@ -21551,28 +21553,28 @@
       <c r="L23" s="37"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A24" s="15" t="s">
+      <c r="A24" s="51" t="s">
         <v>478</v>
       </c>
-      <c r="B24" s="16"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="39"/>
-      <c r="E24" s="40"/>
-      <c r="F24" s="41"/>
-      <c r="G24" s="46"/>
-      <c r="H24" s="47"/>
-      <c r="I24" s="46"/>
-      <c r="J24" s="47"/>
-      <c r="K24" s="46"/>
-      <c r="L24" s="48"/>
+      <c r="B24" s="52"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="29"/>
+      <c r="H24" s="30"/>
+      <c r="I24" s="29"/>
+      <c r="J24" s="30"/>
+      <c r="K24" s="29"/>
+      <c r="L24" s="35"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A25" s="17"/>
-      <c r="B25" s="16"/>
-      <c r="C25" s="39"/>
-      <c r="D25" s="39"/>
-      <c r="E25" s="42"/>
-      <c r="F25" s="43"/>
+      <c r="A25" s="53"/>
+      <c r="B25" s="52"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="26"/>
       <c r="G25" s="31"/>
       <c r="H25" s="32"/>
       <c r="I25" s="31"/>
@@ -21581,12 +21583,12 @@
       <c r="L25" s="36"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A26" s="17"/>
-      <c r="B26" s="16"/>
-      <c r="C26" s="39"/>
-      <c r="D26" s="39"/>
-      <c r="E26" s="44"/>
-      <c r="F26" s="45"/>
+      <c r="A26" s="53"/>
+      <c r="B26" s="52"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="28"/>
       <c r="G26" s="33"/>
       <c r="H26" s="34"/>
       <c r="I26" s="33"/>
@@ -21595,28 +21597,28 @@
       <c r="L26" s="37"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A27" s="15" t="s">
+      <c r="A27" s="51" t="s">
         <v>479</v>
       </c>
-      <c r="B27" s="16"/>
-      <c r="C27" s="38"/>
-      <c r="D27" s="39"/>
-      <c r="E27" s="40"/>
-      <c r="F27" s="41"/>
-      <c r="G27" s="46"/>
-      <c r="H27" s="47"/>
-      <c r="I27" s="46"/>
-      <c r="J27" s="47"/>
-      <c r="K27" s="46"/>
-      <c r="L27" s="48"/>
+      <c r="B27" s="52"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="29"/>
+      <c r="H27" s="30"/>
+      <c r="I27" s="29"/>
+      <c r="J27" s="30"/>
+      <c r="K27" s="29"/>
+      <c r="L27" s="35"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A28" s="17"/>
-      <c r="B28" s="16"/>
-      <c r="C28" s="39"/>
-      <c r="D28" s="39"/>
-      <c r="E28" s="42"/>
-      <c r="F28" s="43"/>
+      <c r="A28" s="53"/>
+      <c r="B28" s="52"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="26"/>
       <c r="G28" s="31"/>
       <c r="H28" s="32"/>
       <c r="I28" s="31"/>
@@ -21625,12 +21627,12 @@
       <c r="L28" s="36"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A29" s="17"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="39"/>
-      <c r="D29" s="39"/>
-      <c r="E29" s="44"/>
-      <c r="F29" s="45"/>
+      <c r="A29" s="53"/>
+      <c r="B29" s="52"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="28"/>
       <c r="G29" s="33"/>
       <c r="H29" s="34"/>
       <c r="I29" s="33"/>
@@ -21639,30 +21641,30 @@
       <c r="L29" s="37"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A30" s="15" t="s">
+      <c r="A30" s="51" t="s">
         <v>480</v>
       </c>
-      <c r="B30" s="16"/>
-      <c r="C30" s="38" t="s">
+      <c r="B30" s="52"/>
+      <c r="C30" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="D30" s="39"/>
-      <c r="E30" s="40"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="46"/>
-      <c r="H30" s="47"/>
-      <c r="I30" s="46"/>
-      <c r="J30" s="47"/>
-      <c r="K30" s="46"/>
-      <c r="L30" s="48"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="29"/>
+      <c r="H30" s="30"/>
+      <c r="I30" s="29"/>
+      <c r="J30" s="30"/>
+      <c r="K30" s="29"/>
+      <c r="L30" s="35"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A31" s="17"/>
-      <c r="B31" s="16"/>
-      <c r="C31" s="39"/>
-      <c r="D31" s="39"/>
-      <c r="E31" s="42"/>
-      <c r="F31" s="43"/>
+      <c r="A31" s="53"/>
+      <c r="B31" s="52"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="25"/>
+      <c r="F31" s="26"/>
       <c r="G31" s="31"/>
       <c r="H31" s="32"/>
       <c r="I31" s="31"/>
@@ -21671,77 +21673,21 @@
       <c r="L31" s="36"/>
     </row>
     <row r="32" spans="1:12" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="18"/>
-      <c r="B32" s="19"/>
-      <c r="C32" s="53"/>
-      <c r="D32" s="53"/>
-      <c r="E32" s="54"/>
-      <c r="F32" s="55"/>
-      <c r="G32" s="56"/>
-      <c r="H32" s="57"/>
-      <c r="I32" s="56"/>
-      <c r="J32" s="57"/>
-      <c r="K32" s="56"/>
-      <c r="L32" s="58"/>
+      <c r="A32" s="54"/>
+      <c r="B32" s="55"/>
+      <c r="C32" s="38"/>
+      <c r="D32" s="38"/>
+      <c r="E32" s="39"/>
+      <c r="F32" s="40"/>
+      <c r="G32" s="41"/>
+      <c r="H32" s="42"/>
+      <c r="I32" s="41"/>
+      <c r="J32" s="42"/>
+      <c r="K32" s="41"/>
+      <c r="L32" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="67">
-    <mergeCell ref="C1:L1"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="C27:D29"/>
-    <mergeCell ref="E27:F29"/>
-    <mergeCell ref="G27:H29"/>
-    <mergeCell ref="I27:J29"/>
-    <mergeCell ref="K27:L29"/>
-    <mergeCell ref="C30:D32"/>
-    <mergeCell ref="E30:F32"/>
-    <mergeCell ref="G30:H32"/>
-    <mergeCell ref="I30:J32"/>
-    <mergeCell ref="K30:L32"/>
-    <mergeCell ref="C21:D23"/>
-    <mergeCell ref="E21:F23"/>
-    <mergeCell ref="G21:H23"/>
-    <mergeCell ref="I21:J23"/>
-    <mergeCell ref="K21:L23"/>
-    <mergeCell ref="C24:D26"/>
-    <mergeCell ref="E24:F26"/>
-    <mergeCell ref="G24:H26"/>
-    <mergeCell ref="I24:J26"/>
-    <mergeCell ref="K24:L26"/>
-    <mergeCell ref="C15:D17"/>
-    <mergeCell ref="E15:F17"/>
-    <mergeCell ref="G15:H17"/>
-    <mergeCell ref="I15:J17"/>
-    <mergeCell ref="K15:L17"/>
-    <mergeCell ref="C18:D20"/>
-    <mergeCell ref="E18:F20"/>
-    <mergeCell ref="G18:H20"/>
-    <mergeCell ref="I18:J20"/>
-    <mergeCell ref="K18:L20"/>
-    <mergeCell ref="E9:F11"/>
-    <mergeCell ref="G9:H11"/>
-    <mergeCell ref="I9:J11"/>
-    <mergeCell ref="K9:L11"/>
-    <mergeCell ref="C12:D14"/>
-    <mergeCell ref="E12:F14"/>
-    <mergeCell ref="G12:H14"/>
-    <mergeCell ref="I12:J14"/>
-    <mergeCell ref="K12:L14"/>
-    <mergeCell ref="C9:D11"/>
-    <mergeCell ref="I3:J5"/>
-    <mergeCell ref="K3:L5"/>
-    <mergeCell ref="C6:D8"/>
-    <mergeCell ref="E6:F8"/>
-    <mergeCell ref="G6:H8"/>
-    <mergeCell ref="I6:J8"/>
-    <mergeCell ref="K6:L8"/>
-    <mergeCell ref="C3:D5"/>
-    <mergeCell ref="E3:F5"/>
-    <mergeCell ref="G3:H5"/>
     <mergeCell ref="A30:B32"/>
     <mergeCell ref="A1:B2"/>
     <mergeCell ref="A3:B5"/>
@@ -21753,6 +21699,62 @@
     <mergeCell ref="A21:B23"/>
     <mergeCell ref="A24:B26"/>
     <mergeCell ref="A27:B29"/>
+    <mergeCell ref="I3:J5"/>
+    <mergeCell ref="K3:L5"/>
+    <mergeCell ref="C6:D8"/>
+    <mergeCell ref="E6:F8"/>
+    <mergeCell ref="G6:H8"/>
+    <mergeCell ref="I6:J8"/>
+    <mergeCell ref="K6:L8"/>
+    <mergeCell ref="C3:D5"/>
+    <mergeCell ref="E3:F5"/>
+    <mergeCell ref="G3:H5"/>
+    <mergeCell ref="E9:F11"/>
+    <mergeCell ref="G9:H11"/>
+    <mergeCell ref="I9:J11"/>
+    <mergeCell ref="K9:L11"/>
+    <mergeCell ref="C12:D14"/>
+    <mergeCell ref="E12:F14"/>
+    <mergeCell ref="G12:H14"/>
+    <mergeCell ref="I12:J14"/>
+    <mergeCell ref="K12:L14"/>
+    <mergeCell ref="C9:D11"/>
+    <mergeCell ref="C18:D20"/>
+    <mergeCell ref="E18:F20"/>
+    <mergeCell ref="G18:H20"/>
+    <mergeCell ref="I18:J20"/>
+    <mergeCell ref="K18:L20"/>
+    <mergeCell ref="C15:D17"/>
+    <mergeCell ref="E15:F17"/>
+    <mergeCell ref="G15:H17"/>
+    <mergeCell ref="I15:J17"/>
+    <mergeCell ref="K15:L17"/>
+    <mergeCell ref="C24:D26"/>
+    <mergeCell ref="E24:F26"/>
+    <mergeCell ref="G24:H26"/>
+    <mergeCell ref="I24:J26"/>
+    <mergeCell ref="K24:L26"/>
+    <mergeCell ref="C21:D23"/>
+    <mergeCell ref="E21:F23"/>
+    <mergeCell ref="G21:H23"/>
+    <mergeCell ref="I21:J23"/>
+    <mergeCell ref="K21:L23"/>
+    <mergeCell ref="C30:D32"/>
+    <mergeCell ref="E30:F32"/>
+    <mergeCell ref="G30:H32"/>
+    <mergeCell ref="I30:J32"/>
+    <mergeCell ref="K30:L32"/>
+    <mergeCell ref="C27:D29"/>
+    <mergeCell ref="E27:F29"/>
+    <mergeCell ref="G27:H29"/>
+    <mergeCell ref="I27:J29"/>
+    <mergeCell ref="K27:L29"/>
+    <mergeCell ref="C1:L1"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="K2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -22488,6 +22490,643 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92F80ACB-A114-4071-ACAA-8FF4763994CA}">
+  <dimension ref="A1:E33"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.6640625" style="3"/>
+    <col min="2" max="2" width="11.1640625" customWidth="1"/>
+    <col min="3" max="3" width="8.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>571</v>
+      </c>
+      <c r="C2" s="13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>571</v>
+      </c>
+      <c r="C3" s="13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>573</v>
+      </c>
+      <c r="C4" s="13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>572</v>
+      </c>
+      <c r="C5" s="13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>571</v>
+      </c>
+      <c r="C6" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D6" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>571</v>
+      </c>
+      <c r="C7" s="13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>572</v>
+      </c>
+      <c r="C8" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D8" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>572</v>
+      </c>
+      <c r="C9" s="13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>571</v>
+      </c>
+      <c r="C10" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D10" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>573</v>
+      </c>
+      <c r="C11" s="13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="3">
+        <v>11</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>572</v>
+      </c>
+      <c r="C12" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D12" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="3">
+        <v>12</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>574</v>
+      </c>
+      <c r="C13" s="13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="3">
+        <v>13</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>572</v>
+      </c>
+      <c r="C14" s="13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="3">
+        <v>14</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>573</v>
+      </c>
+      <c r="C15" s="13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="3">
+        <v>15</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>574</v>
+      </c>
+      <c r="C16" s="13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="3">
+        <v>16</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>574</v>
+      </c>
+      <c r="C17" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="3">
+        <v>17</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>571</v>
+      </c>
+      <c r="C18" s="13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" s="3">
+        <v>18</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>573</v>
+      </c>
+      <c r="C19" s="13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="3">
+        <v>19</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>571</v>
+      </c>
+      <c r="C20" s="13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="3">
+        <v>20</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>572</v>
+      </c>
+      <c r="C21" s="13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="3">
+        <v>21</v>
+      </c>
+      <c r="B22" s="11"/>
+      <c r="C22" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E22" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="3">
+        <v>22</v>
+      </c>
+      <c r="B23" s="11"/>
+      <c r="C23" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="3">
+        <v>23</v>
+      </c>
+      <c r="B24" s="11"/>
+      <c r="C24" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" s="3">
+        <v>24</v>
+      </c>
+      <c r="B25" s="11"/>
+      <c r="C25" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" s="3">
+        <v>25</v>
+      </c>
+      <c r="B26" s="11"/>
+      <c r="C26" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" s="3">
+        <v>26</v>
+      </c>
+      <c r="B27" s="11"/>
+      <c r="C27" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" s="3">
+        <v>27</v>
+      </c>
+      <c r="B28" s="11"/>
+      <c r="C28" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B29" s="11"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B30" s="11"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B31" s="11"/>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B33" t="s">
+        <v>568</v>
+      </c>
+      <c r="C33" s="8">
+        <f>(C2+C3+C4+C5+C6+C7+C8+C9+C10+C11+C12+C13+C14+C15+C16+C17+C18+C19+C20+C21)/20</f>
+        <v>0.75</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94F88A58-2ED9-44A7-B7C0-720CB5D43460}">
+  <dimension ref="A1:E33"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.6640625" style="3"/>
+    <col min="2" max="2" width="11.1640625" customWidth="1"/>
+    <col min="3" max="3" width="8.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="11"/>
+      <c r="C2" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="11"/>
+      <c r="C3" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="11"/>
+      <c r="C4" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="11"/>
+      <c r="C5" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="11"/>
+      <c r="C6" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="11"/>
+      <c r="C7" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="11"/>
+      <c r="C8" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="11"/>
+      <c r="C9" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="11"/>
+      <c r="C10" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="11"/>
+      <c r="C11" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="3">
+        <v>11</v>
+      </c>
+      <c r="B12" s="11"/>
+      <c r="C12" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="3">
+        <v>12</v>
+      </c>
+      <c r="B13" s="11"/>
+      <c r="C13" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="3">
+        <v>13</v>
+      </c>
+      <c r="B14" s="11"/>
+      <c r="C14" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="3">
+        <v>14</v>
+      </c>
+      <c r="B15" s="11"/>
+      <c r="C15" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="3">
+        <v>15</v>
+      </c>
+      <c r="B16" s="11"/>
+      <c r="C16" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="3">
+        <v>16</v>
+      </c>
+      <c r="B17" s="11"/>
+      <c r="C17" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="3">
+        <v>17</v>
+      </c>
+      <c r="B18" s="11"/>
+      <c r="C18" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" s="3">
+        <v>18</v>
+      </c>
+      <c r="B19" s="11"/>
+      <c r="C19" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="3">
+        <v>19</v>
+      </c>
+      <c r="B20" s="11"/>
+      <c r="C20" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="3">
+        <v>20</v>
+      </c>
+      <c r="B21" s="11"/>
+      <c r="C21" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="3">
+        <v>21</v>
+      </c>
+      <c r="B22" s="11"/>
+      <c r="C22" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E22" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="3">
+        <v>22</v>
+      </c>
+      <c r="B23" s="11"/>
+      <c r="C23" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="3">
+        <v>23</v>
+      </c>
+      <c r="B24" s="11"/>
+      <c r="C24" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" s="3">
+        <v>24</v>
+      </c>
+      <c r="B25" s="11"/>
+      <c r="C25" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" s="3">
+        <v>25</v>
+      </c>
+      <c r="B26" s="11"/>
+      <c r="C26" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" s="3">
+        <v>26</v>
+      </c>
+      <c r="B27" s="11"/>
+      <c r="C27" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" s="3">
+        <v>27</v>
+      </c>
+      <c r="B28" s="11"/>
+      <c r="C28" s="13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B29" s="11"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B30" s="11"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B31" s="11"/>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B33" t="s">
+        <v>568</v>
+      </c>
+      <c r="C33" s="8">
+        <f>(C2+C3+C4+C5+C6+C7+C8+C9+C10+C11+C12+C13+C14+C15+C16+C17+C18+C19+C20+C21+C22)/21</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FB16FBF-CE85-40A8-81C5-66FA99BC879C}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>

</xml_diff>